<commit_message>
Chiarisce import Excel e compatta filtri chat app
</commit_message>
<xml_diff>
--- a/public/templates/vygo-import-anagrafiche.xlsx
+++ b/public/templates/vygo-import-anagrafiche.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGGIMI" sheetId="1" r:id="R4447e64cdb0044b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autisti" sheetId="2" r:id="Rd905127519db4f7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone" sheetId="3" r:id="Ra0b1662d7c404a04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mezzi" sheetId="4" r:id="R32da21e28d874abe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrezzature" sheetId="5" r:id="R19091848a062425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenti autisti" sheetId="6" r:id="R2cadfe6059f74cce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scadenze" sheetId="7" r:id="R049974ab54884346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGGIMI" sheetId="1" r:id="R1b9db92d875c42db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autisti" sheetId="2" r:id="R3f85fe4ee0ba4457"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone" sheetId="3" r:id="Ra4dd991a72c24f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mezzi" sheetId="4" r:id="Raea6b97d78374910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrezzature" sheetId="5" r:id="Rdafaa965b6e443db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenti autisti" sheetId="6" r:id="Rab9ad5692029472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scadenze" sheetId="7" r:id="Rdeacfb7c719c499b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,7 +60,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +85,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF97316"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -184,7 +189,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="92">
+  <x:cellXfs count="95">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -301,7 +306,13 @@
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -342,7 +353,10 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -414,10 +428,10 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VygoAutisti" displayName="VygoAutisti" ref="A1:L12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:L12"/>
   <x:tableColumns count="12">
-    <x:tableColumn id="1" name="Nome e cognome"/>
-    <x:tableColumn id="2" name="Username"/>
-    <x:tableColumn id="3" name="Password"/>
-    <x:tableColumn id="4" name="Telefono"/>
+    <x:tableColumn id="1" name="Nome e cognome *"/>
+    <x:tableColumn id="2" name="Username *"/>
+    <x:tableColumn id="3" name="Password *"/>
+    <x:tableColumn id="4" name="Telefono *"/>
     <x:tableColumn id="5" name="Email"/>
     <x:tableColumn id="6" name="Ruolo"/>
     <x:tableColumn id="7" name="Deposito / sede"/>
@@ -435,9 +449,9 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="VygoPersone" displayName="VygoPersone" ref="A1:J12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:J12"/>
   <x:tableColumns count="10">
-    <x:tableColumn id="1" name="Nome e cognome"/>
-    <x:tableColumn id="2" name="Username"/>
-    <x:tableColumn id="3" name="Password"/>
+    <x:tableColumn id="1" name="Nome e cognome *"/>
+    <x:tableColumn id="2" name="Username *"/>
+    <x:tableColumn id="3" name="Password *"/>
     <x:tableColumn id="4" name="Telefono"/>
     <x:tableColumn id="5" name="Email"/>
     <x:tableColumn id="6" name="Reparto"/>
@@ -454,7 +468,7 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VygoMezzi" displayName="VygoMezzi" ref="A1:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G12"/>
   <x:tableColumns count="7">
-    <x:tableColumn id="1" name="Targa"/>
+    <x:tableColumn id="1" name="Targa *"/>
     <x:tableColumn id="2" name="Categoria mezzo"/>
     <x:tableColumn id="3" name="Modello"/>
     <x:tableColumn id="4" name="Allestimento"/>
@@ -470,7 +484,7 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="VygoAttrezzature" displayName="VygoAttrezzature" ref="A1:F12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:F12"/>
   <x:tableColumns count="6">
-    <x:tableColumn id="1" name="Codice"/>
+    <x:tableColumn id="1" name="Codice *"/>
     <x:tableColumn id="2" name="Tipo attrezzatura"/>
     <x:tableColumn id="3" name="Modello"/>
     <x:tableColumn id="4" name="Matricola"/>
@@ -485,9 +499,9 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="VygoDocumentiAutisti" displayName="VygoDocumentiAutisti" ref="A1:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G12"/>
   <x:tableColumns count="7">
-    <x:tableColumn id="1" name="Username autista"/>
-    <x:tableColumn id="2" name="Documento"/>
-    <x:tableColumn id="3" name="Scadenza documento"/>
+    <x:tableColumn id="1" name="Username autista *"/>
+    <x:tableColumn id="2" name="Documento *"/>
+    <x:tableColumn id="3" name="Scadenza documento *"/>
     <x:tableColumn id="4" name="Numero documento"/>
     <x:tableColumn id="5" name="Visibile in app"/>
     <x:tableColumn id="6" name="Responsabile"/>
@@ -501,10 +515,10 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="VygoScadenze" displayName="VygoScadenze" ref="A1:H12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:H12"/>
   <x:tableColumns count="8">
-    <x:tableColumn id="1" name="Ambito scadenza"/>
-    <x:tableColumn id="2" name="Username o targa o codice"/>
-    <x:tableColumn id="3" name="Tipo scadenza"/>
-    <x:tableColumn id="4" name="Data scadenza"/>
+    <x:tableColumn id="1" name="Ambito scadenza *"/>
+    <x:tableColumn id="2" name="Username o targa o codice *"/>
+    <x:tableColumn id="3" name="Tipo scadenza *"/>
+    <x:tableColumn id="4" name="Data scadenza *"/>
     <x:tableColumn id="5" name="Numero documento"/>
     <x:tableColumn id="6" name="Responsabile"/>
     <x:tableColumn id="7" name="Visibile in app"/>
@@ -755,7 +769,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" s="30" t="str">
-        <x:v>Non cambiare i titoli della prima riga: Vygo li usa per capire cosa importare.</x:v>
+        <x:v>I titoli con * e colore arancio sono obbligatori. Gli altri campi sono facoltativi o servono solo se vuoi gia caricare documenti/scadenze.</x:v>
       </x:c>
       <x:c r="C5" s="30" t="str"/>
       <x:c r="D5" s="30" t="str"/>
@@ -769,7 +783,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B6" s="30" t="str">
-        <x:v>Le date possono essere scritte come 2027-05-31 oppure 31/05/2027.</x:v>
+        <x:v>Non cambiare i titoli della prima riga: Vygo li usa per capire cosa importare.</x:v>
       </x:c>
       <x:c r="C6" s="30" t="str"/>
       <x:c r="D6" s="30" t="str"/>
@@ -783,7 +797,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B7" s="30" t="str">
-        <x:v>Username, targhe e codici devono essere unici. Se li ripeti, Vygo ti segnala l errore prima di importare.</x:v>
+        <x:v>Le date possono essere scritte come 2027-05-31 oppure 31/05/2027.</x:v>
       </x:c>
       <x:c r="C7" s="30" t="str"/>
       <x:c r="D7" s="30" t="str"/>
@@ -880,374 +894,374 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="69" t="str">
-        <x:v>Nome e cognome</x:v>
-      </x:c>
-      <x:c r="B1" s="70" t="str">
-        <x:v>Username</x:v>
-      </x:c>
-      <x:c r="C1" s="70" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="D1" s="70" t="str">
-        <x:v>Telefono</x:v>
-      </x:c>
-      <x:c r="E1" s="70" t="str">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Nome e cognome *</x:v>
+      </x:c>
+      <x:c r="B1" s="72" t="str">
+        <x:v>Username *</x:v>
+      </x:c>
+      <x:c r="C1" s="72" t="str">
+        <x:v>Password *</x:v>
+      </x:c>
+      <x:c r="D1" s="72" t="str">
+        <x:v>Telefono *</x:v>
+      </x:c>
+      <x:c r="E1" s="73" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="F1" s="70" t="str">
+      <x:c r="F1" s="73" t="str">
         <x:v>Ruolo</x:v>
       </x:c>
-      <x:c r="G1" s="70" t="str">
+      <x:c r="G1" s="73" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="H1" s="70" t="str">
+      <x:c r="H1" s="73" t="str">
         <x:v>Documento iniziale</x:v>
       </x:c>
-      <x:c r="I1" s="70" t="str">
+      <x:c r="I1" s="73" t="str">
         <x:v>Scadenza documento</x:v>
       </x:c>
-      <x:c r="J1" s="70" t="str">
+      <x:c r="J1" s="73" t="str">
         <x:v>Numero documento</x:v>
       </x:c>
-      <x:c r="K1" s="70" t="str">
+      <x:c r="K1" s="73" t="str">
         <x:v>Visibile in app</x:v>
       </x:c>
-      <x:c r="L1" s="71" t="str">
+      <x:c r="L1" s="74" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="72" t="str">
+      <x:c r="A2" s="75" t="str">
         <x:v>Mario Rossi</x:v>
       </x:c>
-      <x:c r="B2" s="73" t="str">
+      <x:c r="B2" s="76" t="str">
         <x:v>mario.rossi</x:v>
       </x:c>
-      <x:c r="C2" s="73" t="str">
+      <x:c r="C2" s="76" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D2" s="73" t="str">
+      <x:c r="D2" s="76" t="str">
         <x:v>+39 333 111 1111</x:v>
       </x:c>
-      <x:c r="E2" s="74" t="str">
+      <x:c r="E2" s="77" t="str">
         <x:v>mario.rossi@azienda.it</x:v>
       </x:c>
-      <x:c r="F2" s="74" t="str">
+      <x:c r="F2" s="77" t="str">
         <x:v>Autista bilico</x:v>
       </x:c>
-      <x:c r="G2" s="74" t="str">
+      <x:c r="G2" s="77" t="str">
         <x:v>Verona</x:v>
       </x:c>
-      <x:c r="H2" s="74" t="str">
+      <x:c r="H2" s="77" t="str">
         <x:v>Patente C+E</x:v>
       </x:c>
-      <x:c r="I2" s="89" t="str">
+      <x:c r="I2" s="92" t="str">
         <x:v>2027-05-31</x:v>
       </x:c>
-      <x:c r="J2" s="73" t="str">
+      <x:c r="J2" s="76" t="str">
         <x:v>PCE12345</x:v>
       </x:c>
-      <x:c r="K2" s="74" t="str">
+      <x:c r="K2" s="77" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="L2" s="75" t="str">
+      <x:c r="L2" s="78" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="76" t="str">
+      <x:c r="A3" s="79" t="str">
         <x:v>Anna Verdi</x:v>
       </x:c>
-      <x:c r="B3" s="77" t="str">
+      <x:c r="B3" s="80" t="str">
         <x:v>anna.verdi</x:v>
       </x:c>
-      <x:c r="C3" s="77" t="str">
+      <x:c r="C3" s="80" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D3" s="77" t="str">
+      <x:c r="D3" s="80" t="str">
         <x:v>+39 333 222 2222</x:v>
       </x:c>
-      <x:c r="E3" s="78" t="str">
+      <x:c r="E3" s="81" t="str">
         <x:v>anna.verdi@azienda.it</x:v>
       </x:c>
-      <x:c r="F3" s="78" t="str">
+      <x:c r="F3" s="81" t="str">
         <x:v>Autista furgone</x:v>
       </x:c>
-      <x:c r="G3" s="78" t="str">
+      <x:c r="G3" s="81" t="str">
         <x:v>Milano</x:v>
       </x:c>
-      <x:c r="H3" s="78" t="str">
+      <x:c r="H3" s="81" t="str">
         <x:v>CQC</x:v>
       </x:c>
-      <x:c r="I3" s="90" t="str">
+      <x:c r="I3" s="93" t="str">
         <x:v>2027-11-30</x:v>
       </x:c>
-      <x:c r="J3" s="77" t="str">
+      <x:c r="J3" s="80" t="str">
         <x:v>CQC9988</x:v>
       </x:c>
-      <x:c r="K3" s="78" t="str">
+      <x:c r="K3" s="81" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="L3" s="79" t="str"/>
+      <x:c r="L3" s="82" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="B4" s="45"/>
       <x:c r="C4" s="45"/>
       <x:c r="D4" s="45"/>
-      <x:c r="I4" s="91"/>
+      <x:c r="I4" s="94"/>
       <x:c r="J4" s="45"/>
     </x:row>
     <x:row r="5">
       <x:c r="B5" s="45"/>
       <x:c r="C5" s="45"/>
       <x:c r="D5" s="45"/>
-      <x:c r="I5" s="91"/>
+      <x:c r="I5" s="94"/>
       <x:c r="J5" s="45"/>
     </x:row>
     <x:row r="6">
       <x:c r="B6" s="45"/>
       <x:c r="C6" s="45"/>
       <x:c r="D6" s="45"/>
-      <x:c r="I6" s="91"/>
+      <x:c r="I6" s="94"/>
       <x:c r="J6" s="45"/>
     </x:row>
     <x:row r="7">
       <x:c r="B7" s="45"/>
       <x:c r="C7" s="45"/>
       <x:c r="D7" s="45"/>
-      <x:c r="I7" s="91"/>
+      <x:c r="I7" s="94"/>
       <x:c r="J7" s="45"/>
     </x:row>
     <x:row r="8">
       <x:c r="B8" s="45"/>
       <x:c r="C8" s="45"/>
       <x:c r="D8" s="45"/>
-      <x:c r="I8" s="91"/>
+      <x:c r="I8" s="94"/>
       <x:c r="J8" s="45"/>
     </x:row>
     <x:row r="9">
       <x:c r="B9" s="45"/>
       <x:c r="C9" s="45"/>
       <x:c r="D9" s="45"/>
-      <x:c r="I9" s="91"/>
+      <x:c r="I9" s="94"/>
       <x:c r="J9" s="45"/>
     </x:row>
     <x:row r="10">
       <x:c r="B10" s="45"/>
       <x:c r="C10" s="45"/>
       <x:c r="D10" s="45"/>
-      <x:c r="I10" s="91"/>
+      <x:c r="I10" s="94"/>
       <x:c r="J10" s="45"/>
     </x:row>
     <x:row r="11">
       <x:c r="B11" s="45"/>
       <x:c r="C11" s="45"/>
       <x:c r="D11" s="45"/>
-      <x:c r="I11" s="91"/>
+      <x:c r="I11" s="94"/>
       <x:c r="J11" s="45"/>
     </x:row>
     <x:row r="12">
       <x:c r="B12" s="45"/>
       <x:c r="C12" s="45"/>
       <x:c r="D12" s="45"/>
-      <x:c r="I12" s="91"/>
+      <x:c r="I12" s="94"/>
       <x:c r="J12" s="45"/>
     </x:row>
     <x:row r="13">
       <x:c r="B13" s="45"/>
       <x:c r="C13" s="45"/>
       <x:c r="D13" s="45"/>
-      <x:c r="I13" s="91"/>
+      <x:c r="I13" s="94"/>
       <x:c r="J13" s="45"/>
     </x:row>
     <x:row r="14">
       <x:c r="B14" s="45"/>
       <x:c r="C14" s="45"/>
       <x:c r="D14" s="45"/>
-      <x:c r="I14" s="91"/>
+      <x:c r="I14" s="94"/>
       <x:c r="J14" s="45"/>
     </x:row>
     <x:row r="15">
       <x:c r="B15" s="45"/>
       <x:c r="C15" s="45"/>
       <x:c r="D15" s="45"/>
-      <x:c r="I15" s="91"/>
+      <x:c r="I15" s="94"/>
       <x:c r="J15" s="45"/>
     </x:row>
     <x:row r="16">
       <x:c r="B16" s="45"/>
       <x:c r="C16" s="45"/>
       <x:c r="D16" s="45"/>
-      <x:c r="I16" s="91"/>
+      <x:c r="I16" s="94"/>
       <x:c r="J16" s="45"/>
     </x:row>
     <x:row r="17">
       <x:c r="B17" s="45"/>
       <x:c r="C17" s="45"/>
       <x:c r="D17" s="45"/>
-      <x:c r="I17" s="91"/>
+      <x:c r="I17" s="94"/>
       <x:c r="J17" s="45"/>
     </x:row>
     <x:row r="18">
       <x:c r="B18" s="45"/>
       <x:c r="C18" s="45"/>
       <x:c r="D18" s="45"/>
-      <x:c r="I18" s="91"/>
+      <x:c r="I18" s="94"/>
       <x:c r="J18" s="45"/>
     </x:row>
     <x:row r="19">
       <x:c r="B19" s="45"/>
       <x:c r="C19" s="45"/>
       <x:c r="D19" s="45"/>
-      <x:c r="I19" s="91"/>
+      <x:c r="I19" s="94"/>
       <x:c r="J19" s="45"/>
     </x:row>
     <x:row r="20">
       <x:c r="B20" s="45"/>
       <x:c r="C20" s="45"/>
       <x:c r="D20" s="45"/>
-      <x:c r="I20" s="91"/>
+      <x:c r="I20" s="94"/>
       <x:c r="J20" s="45"/>
     </x:row>
     <x:row r="21">
       <x:c r="B21" s="45"/>
       <x:c r="C21" s="45"/>
       <x:c r="D21" s="45"/>
-      <x:c r="I21" s="91"/>
+      <x:c r="I21" s="94"/>
       <x:c r="J21" s="45"/>
     </x:row>
     <x:row r="22">
       <x:c r="B22" s="45"/>
       <x:c r="C22" s="45"/>
       <x:c r="D22" s="45"/>
-      <x:c r="I22" s="91"/>
+      <x:c r="I22" s="94"/>
       <x:c r="J22" s="45"/>
     </x:row>
     <x:row r="23">
       <x:c r="B23" s="45"/>
       <x:c r="C23" s="45"/>
       <x:c r="D23" s="45"/>
-      <x:c r="I23" s="91"/>
+      <x:c r="I23" s="94"/>
       <x:c r="J23" s="45"/>
     </x:row>
     <x:row r="24">
       <x:c r="B24" s="45"/>
       <x:c r="C24" s="45"/>
       <x:c r="D24" s="45"/>
-      <x:c r="I24" s="91"/>
+      <x:c r="I24" s="94"/>
       <x:c r="J24" s="45"/>
     </x:row>
     <x:row r="25">
       <x:c r="B25" s="45"/>
       <x:c r="C25" s="45"/>
       <x:c r="D25" s="45"/>
-      <x:c r="I25" s="91"/>
+      <x:c r="I25" s="94"/>
       <x:c r="J25" s="45"/>
     </x:row>
     <x:row r="26">
       <x:c r="B26" s="45"/>
       <x:c r="C26" s="45"/>
       <x:c r="D26" s="45"/>
-      <x:c r="I26" s="91"/>
+      <x:c r="I26" s="94"/>
       <x:c r="J26" s="45"/>
     </x:row>
     <x:row r="27">
       <x:c r="B27" s="45"/>
       <x:c r="C27" s="45"/>
       <x:c r="D27" s="45"/>
-      <x:c r="I27" s="91"/>
+      <x:c r="I27" s="94"/>
       <x:c r="J27" s="45"/>
     </x:row>
     <x:row r="28">
       <x:c r="B28" s="45"/>
       <x:c r="C28" s="45"/>
       <x:c r="D28" s="45"/>
-      <x:c r="I28" s="91"/>
+      <x:c r="I28" s="94"/>
       <x:c r="J28" s="45"/>
     </x:row>
     <x:row r="29">
       <x:c r="B29" s="45"/>
       <x:c r="C29" s="45"/>
       <x:c r="D29" s="45"/>
-      <x:c r="I29" s="91"/>
+      <x:c r="I29" s="94"/>
       <x:c r="J29" s="45"/>
     </x:row>
     <x:row r="30">
       <x:c r="B30" s="45"/>
       <x:c r="C30" s="45"/>
       <x:c r="D30" s="45"/>
-      <x:c r="I30" s="91"/>
+      <x:c r="I30" s="94"/>
       <x:c r="J30" s="45"/>
     </x:row>
     <x:row r="31">
       <x:c r="B31" s="45"/>
       <x:c r="C31" s="45"/>
       <x:c r="D31" s="45"/>
-      <x:c r="I31" s="91"/>
+      <x:c r="I31" s="94"/>
       <x:c r="J31" s="45"/>
     </x:row>
     <x:row r="32">
       <x:c r="B32" s="45"/>
       <x:c r="C32" s="45"/>
       <x:c r="D32" s="45"/>
-      <x:c r="I32" s="91"/>
+      <x:c r="I32" s="94"/>
       <x:c r="J32" s="45"/>
     </x:row>
     <x:row r="33">
       <x:c r="B33" s="45"/>
       <x:c r="C33" s="45"/>
       <x:c r="D33" s="45"/>
-      <x:c r="I33" s="91"/>
+      <x:c r="I33" s="94"/>
       <x:c r="J33" s="45"/>
     </x:row>
     <x:row r="34">
       <x:c r="B34" s="45"/>
       <x:c r="C34" s="45"/>
       <x:c r="D34" s="45"/>
-      <x:c r="I34" s="91"/>
+      <x:c r="I34" s="94"/>
       <x:c r="J34" s="45"/>
     </x:row>
     <x:row r="35">
       <x:c r="B35" s="45"/>
       <x:c r="C35" s="45"/>
       <x:c r="D35" s="45"/>
-      <x:c r="I35" s="91"/>
+      <x:c r="I35" s="94"/>
       <x:c r="J35" s="45"/>
     </x:row>
     <x:row r="36">
       <x:c r="B36" s="45"/>
       <x:c r="C36" s="45"/>
       <x:c r="D36" s="45"/>
-      <x:c r="I36" s="91"/>
+      <x:c r="I36" s="94"/>
       <x:c r="J36" s="45"/>
     </x:row>
     <x:row r="37">
       <x:c r="B37" s="45"/>
       <x:c r="C37" s="45"/>
       <x:c r="D37" s="45"/>
-      <x:c r="I37" s="91"/>
+      <x:c r="I37" s="94"/>
       <x:c r="J37" s="45"/>
     </x:row>
     <x:row r="38">
       <x:c r="B38" s="45"/>
       <x:c r="C38" s="45"/>
       <x:c r="D38" s="45"/>
-      <x:c r="I38" s="91"/>
+      <x:c r="I38" s="94"/>
       <x:c r="J38" s="45"/>
     </x:row>
     <x:row r="39">
       <x:c r="B39" s="45"/>
       <x:c r="C39" s="45"/>
       <x:c r="D39" s="45"/>
-      <x:c r="I39" s="91"/>
+      <x:c r="I39" s="94"/>
       <x:c r="J39" s="45"/>
     </x:row>
     <x:row r="40">
       <x:c r="B40" s="45"/>
       <x:c r="C40" s="45"/>
       <x:c r="D40" s="45"/>
-      <x:c r="I40" s="91"/>
+      <x:c r="I40" s="94"/>
       <x:c r="J40" s="45"/>
     </x:row>
   </x:sheetData>
@@ -1258,7 +1272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbc4baf99bbc4ebd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83883da298bc4138"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1280,98 +1294,98 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="69" t="str">
-        <x:v>Nome e cognome</x:v>
-      </x:c>
-      <x:c r="B1" s="70" t="str">
-        <x:v>Username</x:v>
-      </x:c>
-      <x:c r="C1" s="70" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="D1" s="70" t="str">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Nome e cognome *</x:v>
+      </x:c>
+      <x:c r="B1" s="72" t="str">
+        <x:v>Username *</x:v>
+      </x:c>
+      <x:c r="C1" s="72" t="str">
+        <x:v>Password *</x:v>
+      </x:c>
+      <x:c r="D1" s="73" t="str">
         <x:v>Telefono</x:v>
       </x:c>
-      <x:c r="E1" s="70" t="str">
+      <x:c r="E1" s="73" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="F1" s="70" t="str">
+      <x:c r="F1" s="73" t="str">
         <x:v>Reparto</x:v>
       </x:c>
-      <x:c r="G1" s="70" t="str">
+      <x:c r="G1" s="73" t="str">
         <x:v>Ruolo</x:v>
       </x:c>
-      <x:c r="H1" s="70" t="str">
+      <x:c r="H1" s="73" t="str">
         <x:v>Mansione</x:v>
       </x:c>
-      <x:c r="I1" s="70" t="str">
+      <x:c r="I1" s="73" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="J1" s="71" t="str">
+      <x:c r="J1" s="74" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="72" t="str">
+      <x:c r="A2" s="75" t="str">
         <x:v>Paola Bianchi</x:v>
       </x:c>
-      <x:c r="B2" s="73" t="str">
+      <x:c r="B2" s="76" t="str">
         <x:v>paola.bianchi</x:v>
       </x:c>
-      <x:c r="C2" s="73" t="str">
+      <x:c r="C2" s="76" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D2" s="73" t="str">
+      <x:c r="D2" s="76" t="str">
         <x:v>+39 333 444 4444</x:v>
       </x:c>
-      <x:c r="E2" s="74" t="str">
+      <x:c r="E2" s="77" t="str">
         <x:v>paola.bianchi@azienda.it</x:v>
       </x:c>
-      <x:c r="F2" s="74" t="str">
+      <x:c r="F2" s="77" t="str">
         <x:v>ufficio</x:v>
       </x:c>
-      <x:c r="G2" s="74" t="str">
+      <x:c r="G2" s="77" t="str">
         <x:v>Impiegato ufficio</x:v>
       </x:c>
-      <x:c r="H2" s="74" t="str">
+      <x:c r="H2" s="77" t="str">
         <x:v>Ufficio traffico</x:v>
       </x:c>
-      <x:c r="I2" s="74" t="str">
+      <x:c r="I2" s="77" t="str">
         <x:v>Sede centrale</x:v>
       </x:c>
-      <x:c r="J2" s="75" t="str">
+      <x:c r="J2" s="78" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="76" t="str">
+      <x:c r="A3" s="79" t="str">
         <x:v>Luca Neri</x:v>
       </x:c>
-      <x:c r="B3" s="77" t="str">
+      <x:c r="B3" s="80" t="str">
         <x:v>luca.neri</x:v>
       </x:c>
-      <x:c r="C3" s="77" t="str">
+      <x:c r="C3" s="80" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D3" s="77" t="str">
+      <x:c r="D3" s="80" t="str">
         <x:v>+39 333 555 5555</x:v>
       </x:c>
-      <x:c r="E3" s="78" t="str">
+      <x:c r="E3" s="81" t="str">
         <x:v>luca.neri@azienda.it</x:v>
       </x:c>
-      <x:c r="F3" s="78" t="str">
+      <x:c r="F3" s="81" t="str">
         <x:v>magazzino</x:v>
       </x:c>
-      <x:c r="G3" s="78" t="str">
+      <x:c r="G3" s="81" t="str">
         <x:v>Carrellista</x:v>
       </x:c>
-      <x:c r="H3" s="78" t="str">
+      <x:c r="H3" s="81" t="str">
         <x:v>Capo turno magazzino</x:v>
       </x:c>
-      <x:c r="I3" s="78" t="str">
+      <x:c r="I3" s="81" t="str">
         <x:v>Magazzino A</x:v>
       </x:c>
-      <x:c r="J3" s="79" t="str"/>
+      <x:c r="J3" s="82" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="B4" s="45"/>
@@ -1569,7 +1583,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0901697c6963469e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R271d9229258d40ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1588,236 +1602,236 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="69" t="str">
-        <x:v>Targa</x:v>
-      </x:c>
-      <x:c r="B1" s="70" t="str">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Targa *</x:v>
+      </x:c>
+      <x:c r="B1" s="73" t="str">
         <x:v>Categoria mezzo</x:v>
       </x:c>
-      <x:c r="C1" s="70" t="str">
+      <x:c r="C1" s="73" t="str">
         <x:v>Modello</x:v>
       </x:c>
-      <x:c r="D1" s="70" t="str">
+      <x:c r="D1" s="73" t="str">
         <x:v>Allestimento</x:v>
       </x:c>
-      <x:c r="E1" s="70" t="str">
+      <x:c r="E1" s="73" t="str">
         <x:v>KM</x:v>
       </x:c>
-      <x:c r="F1" s="70" t="str">
+      <x:c r="F1" s="73" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="G1" s="71" t="str">
+      <x:c r="G1" s="74" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="84" t="str">
+      <x:c r="A2" s="87" t="str">
         <x:v>AB123CD</x:v>
       </x:c>
-      <x:c r="B2" s="74" t="str">
+      <x:c r="B2" s="77" t="str">
         <x:v>trattore</x:v>
       </x:c>
-      <x:c r="C2" s="74" t="str">
+      <x:c r="C2" s="77" t="str">
         <x:v>Volvo FH</x:v>
       </x:c>
-      <x:c r="D2" s="74" t="str">
+      <x:c r="D2" s="77" t="str">
         <x:v>Trattore stradale</x:v>
       </x:c>
-      <x:c r="E2" s="86" t="n">
+      <x:c r="E2" s="89" t="n">
         <x:v>340000</x:v>
       </x:c>
-      <x:c r="F2" s="74" t="str">
+      <x:c r="F2" s="77" t="str">
         <x:v>Verona</x:v>
       </x:c>
-      <x:c r="G2" s="75" t="str">
+      <x:c r="G2" s="78" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="84" t="str">
+      <x:c r="A3" s="87" t="str">
         <x:v>SR456EF</x:v>
       </x:c>
-      <x:c r="B3" s="74" t="str">
+      <x:c r="B3" s="77" t="str">
         <x:v>semirimorchio</x:v>
       </x:c>
-      <x:c r="C3" s="74" t="str">
+      <x:c r="C3" s="77" t="str">
         <x:v>Krone</x:v>
       </x:c>
-      <x:c r="D3" s="74" t="str">
+      <x:c r="D3" s="77" t="str">
         <x:v>Centinato</x:v>
       </x:c>
-      <x:c r="E3" s="86" t="n">
+      <x:c r="E3" s="89" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F3" s="74" t="str">
+      <x:c r="F3" s="77" t="str">
         <x:v>Verona</x:v>
       </x:c>
-      <x:c r="G3" s="75" t="str"/>
+      <x:c r="G3" s="78" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="85" t="str">
+      <x:c r="A4" s="88" t="str">
         <x:v>FG789HI</x:v>
       </x:c>
-      <x:c r="B4" s="78" t="str">
+      <x:c r="B4" s="81" t="str">
         <x:v>furgone</x:v>
       </x:c>
-      <x:c r="C4" s="78" t="str">
+      <x:c r="C4" s="81" t="str">
         <x:v>Iveco Daily</x:v>
       </x:c>
-      <x:c r="D4" s="78" t="str">
+      <x:c r="D4" s="81" t="str">
         <x:v>Furgone cassonato</x:v>
       </x:c>
-      <x:c r="E4" s="87" t="n">
+      <x:c r="E4" s="90" t="n">
         <x:v>82000</x:v>
       </x:c>
-      <x:c r="F4" s="78" t="str">
+      <x:c r="F4" s="81" t="str">
         <x:v>Milano</x:v>
       </x:c>
-      <x:c r="G4" s="79" t="str"/>
+      <x:c r="G4" s="82" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="45"/>
-      <x:c r="E5" s="88"/>
+      <x:c r="E5" s="91"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="45"/>
-      <x:c r="E6" s="88"/>
+      <x:c r="E6" s="91"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="45"/>
-      <x:c r="E7" s="88"/>
+      <x:c r="E7" s="91"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="45"/>
-      <x:c r="E8" s="88"/>
+      <x:c r="E8" s="91"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="45"/>
-      <x:c r="E9" s="88"/>
+      <x:c r="E9" s="91"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="45"/>
-      <x:c r="E10" s="88"/>
+      <x:c r="E10" s="91"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="45"/>
-      <x:c r="E11" s="88"/>
+      <x:c r="E11" s="91"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45"/>
-      <x:c r="E12" s="88"/>
+      <x:c r="E12" s="91"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45"/>
-      <x:c r="E13" s="88"/>
+      <x:c r="E13" s="91"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="45"/>
-      <x:c r="E14" s="88"/>
+      <x:c r="E14" s="91"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="45"/>
-      <x:c r="E15" s="88"/>
+      <x:c r="E15" s="91"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="45"/>
-      <x:c r="E16" s="88"/>
+      <x:c r="E16" s="91"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="45"/>
-      <x:c r="E17" s="88"/>
+      <x:c r="E17" s="91"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="45"/>
-      <x:c r="E18" s="88"/>
+      <x:c r="E18" s="91"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="45"/>
-      <x:c r="E19" s="88"/>
+      <x:c r="E19" s="91"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="45"/>
-      <x:c r="E20" s="88"/>
+      <x:c r="E20" s="91"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="45"/>
-      <x:c r="E21" s="88"/>
+      <x:c r="E21" s="91"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="45"/>
-      <x:c r="E22" s="88"/>
+      <x:c r="E22" s="91"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="45"/>
-      <x:c r="E23" s="88"/>
+      <x:c r="E23" s="91"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="45"/>
-      <x:c r="E24" s="88"/>
+      <x:c r="E24" s="91"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="45"/>
-      <x:c r="E25" s="88"/>
+      <x:c r="E25" s="91"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="45"/>
-      <x:c r="E26" s="88"/>
+      <x:c r="E26" s="91"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="45"/>
-      <x:c r="E27" s="88"/>
+      <x:c r="E27" s="91"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="45"/>
-      <x:c r="E28" s="88"/>
+      <x:c r="E28" s="91"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="45"/>
-      <x:c r="E29" s="88"/>
+      <x:c r="E29" s="91"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="45"/>
-      <x:c r="E30" s="88"/>
+      <x:c r="E30" s="91"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="45"/>
-      <x:c r="E31" s="88"/>
+      <x:c r="E31" s="91"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="45"/>
-      <x:c r="E32" s="88"/>
+      <x:c r="E32" s="91"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="45"/>
-      <x:c r="E33" s="88"/>
+      <x:c r="E33" s="91"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="45"/>
-      <x:c r="E34" s="88"/>
+      <x:c r="E34" s="91"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="45"/>
-      <x:c r="E35" s="88"/>
+      <x:c r="E35" s="91"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="45"/>
-      <x:c r="E36" s="88"/>
+      <x:c r="E36" s="91"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="45"/>
-      <x:c r="E37" s="88"/>
+      <x:c r="E37" s="91"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="45"/>
-      <x:c r="E38" s="88"/>
+      <x:c r="E38" s="91"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="45"/>
-      <x:c r="E39" s="88"/>
+      <x:c r="E39" s="91"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="45"/>
-      <x:c r="E40" s="88"/>
+      <x:c r="E40" s="91"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1827,7 +1841,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re260339827c540f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43c5a6c3ef8a47d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1845,62 +1859,62 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="69" t="str">
-        <x:v>Codice</x:v>
-      </x:c>
-      <x:c r="B1" s="70" t="str">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Codice *</x:v>
+      </x:c>
+      <x:c r="B1" s="73" t="str">
         <x:v>Tipo attrezzatura</x:v>
       </x:c>
-      <x:c r="C1" s="70" t="str">
+      <x:c r="C1" s="73" t="str">
         <x:v>Modello</x:v>
       </x:c>
-      <x:c r="D1" s="70" t="str">
+      <x:c r="D1" s="73" t="str">
         <x:v>Matricola</x:v>
       </x:c>
-      <x:c r="E1" s="70" t="str">
+      <x:c r="E1" s="73" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="F1" s="71" t="str">
+      <x:c r="F1" s="74" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="84" t="str">
+      <x:c r="A2" s="87" t="str">
         <x:v>MUL-01</x:v>
       </x:c>
-      <x:c r="B2" s="73" t="str">
+      <x:c r="B2" s="76" t="str">
         <x:v>muletto</x:v>
       </x:c>
-      <x:c r="C2" s="73" t="str">
+      <x:c r="C2" s="76" t="str">
         <x:v>Toyota 8FB</x:v>
       </x:c>
-      <x:c r="D2" s="73" t="str">
+      <x:c r="D2" s="76" t="str">
         <x:v>MAT-987</x:v>
       </x:c>
-      <x:c r="E2" s="74" t="str">
+      <x:c r="E2" s="77" t="str">
         <x:v>Magazzino A</x:v>
       </x:c>
-      <x:c r="F2" s="75" t="str">
+      <x:c r="F2" s="78" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="85" t="str">
+      <x:c r="A3" s="88" t="str">
         <x:v>TP-02</x:v>
       </x:c>
-      <x:c r="B3" s="77" t="str">
+      <x:c r="B3" s="80" t="str">
         <x:v>transpallet</x:v>
       </x:c>
-      <x:c r="C3" s="77" t="str">
+      <x:c r="C3" s="80" t="str">
         <x:v>BT Levio</x:v>
       </x:c>
-      <x:c r="D3" s="77" t="str">
+      <x:c r="D3" s="80" t="str">
         <x:v>TP-445</x:v>
       </x:c>
-      <x:c r="E3" s="78" t="str">
+      <x:c r="E3" s="81" t="str">
         <x:v>Magazzino A</x:v>
       </x:c>
-      <x:c r="F3" s="79" t="str"/>
+      <x:c r="F3" s="82" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="45"/>
@@ -2132,7 +2146,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0280121e7464348"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R762e134555874c91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2151,255 +2165,255 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="69" t="str">
-        <x:v>Username autista</x:v>
-      </x:c>
-      <x:c r="B1" s="70" t="str">
-        <x:v>Documento</x:v>
-      </x:c>
-      <x:c r="C1" s="70" t="str">
-        <x:v>Scadenza documento</x:v>
-      </x:c>
-      <x:c r="D1" s="70" t="str">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Username autista *</x:v>
+      </x:c>
+      <x:c r="B1" s="72" t="str">
+        <x:v>Documento *</x:v>
+      </x:c>
+      <x:c r="C1" s="72" t="str">
+        <x:v>Scadenza documento *</x:v>
+      </x:c>
+      <x:c r="D1" s="73" t="str">
         <x:v>Numero documento</x:v>
       </x:c>
-      <x:c r="E1" s="70" t="str">
+      <x:c r="E1" s="73" t="str">
         <x:v>Visibile in app</x:v>
       </x:c>
-      <x:c r="F1" s="70" t="str">
+      <x:c r="F1" s="73" t="str">
         <x:v>Responsabile</x:v>
       </x:c>
-      <x:c r="G1" s="71" t="str">
+      <x:c r="G1" s="74" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="84" t="str">
+      <x:c r="A2" s="87" t="str">
         <x:v>mario.rossi</x:v>
       </x:c>
-      <x:c r="B2" s="74" t="str">
+      <x:c r="B2" s="77" t="str">
         <x:v>CQC</x:v>
       </x:c>
-      <x:c r="C2" s="89" t="str">
+      <x:c r="C2" s="92" t="str">
         <x:v>2027-11-30</x:v>
       </x:c>
-      <x:c r="D2" s="73" t="str">
+      <x:c r="D2" s="76" t="str">
         <x:v>CQC9988</x:v>
       </x:c>
-      <x:c r="E2" s="74" t="str">
+      <x:c r="E2" s="77" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="F2" s="74" t="str">
+      <x:c r="F2" s="77" t="str">
         <x:v>Ufficio personale</x:v>
       </x:c>
-      <x:c r="G2" s="75" t="str">
+      <x:c r="G2" s="78" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="85" t="str">
+      <x:c r="A3" s="88" t="str">
         <x:v>anna.verdi</x:v>
       </x:c>
-      <x:c r="B3" s="78" t="str">
+      <x:c r="B3" s="81" t="str">
         <x:v>Visita medica</x:v>
       </x:c>
-      <x:c r="C3" s="90" t="str">
+      <x:c r="C3" s="93" t="str">
         <x:v>2027-04-20</x:v>
       </x:c>
-      <x:c r="D3" s="77" t="str">
+      <x:c r="D3" s="80" t="str">
         <x:v>VM-ANNA</x:v>
       </x:c>
-      <x:c r="E3" s="78" t="str">
+      <x:c r="E3" s="81" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="F3" s="78" t="str">
+      <x:c r="F3" s="81" t="str">
         <x:v>Ufficio personale</x:v>
       </x:c>
-      <x:c r="G3" s="79" t="str"/>
+      <x:c r="G3" s="82" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="45"/>
-      <x:c r="C4" s="91"/>
+      <x:c r="C4" s="94"/>
       <x:c r="D4" s="45"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="45"/>
-      <x:c r="C5" s="91"/>
+      <x:c r="C5" s="94"/>
       <x:c r="D5" s="45"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="45"/>
-      <x:c r="C6" s="91"/>
+      <x:c r="C6" s="94"/>
       <x:c r="D6" s="45"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="45"/>
-      <x:c r="C7" s="91"/>
+      <x:c r="C7" s="94"/>
       <x:c r="D7" s="45"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="45"/>
-      <x:c r="C8" s="91"/>
+      <x:c r="C8" s="94"/>
       <x:c r="D8" s="45"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="45"/>
-      <x:c r="C9" s="91"/>
+      <x:c r="C9" s="94"/>
       <x:c r="D9" s="45"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="45"/>
-      <x:c r="C10" s="91"/>
+      <x:c r="C10" s="94"/>
       <x:c r="D10" s="45"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="45"/>
-      <x:c r="C11" s="91"/>
+      <x:c r="C11" s="94"/>
       <x:c r="D11" s="45"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45"/>
-      <x:c r="C12" s="91"/>
+      <x:c r="C12" s="94"/>
       <x:c r="D12" s="45"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45"/>
-      <x:c r="C13" s="91"/>
+      <x:c r="C13" s="94"/>
       <x:c r="D13" s="45"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="45"/>
-      <x:c r="C14" s="91"/>
+      <x:c r="C14" s="94"/>
       <x:c r="D14" s="45"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="45"/>
-      <x:c r="C15" s="91"/>
+      <x:c r="C15" s="94"/>
       <x:c r="D15" s="45"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="45"/>
-      <x:c r="C16" s="91"/>
+      <x:c r="C16" s="94"/>
       <x:c r="D16" s="45"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="45"/>
-      <x:c r="C17" s="91"/>
+      <x:c r="C17" s="94"/>
       <x:c r="D17" s="45"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="45"/>
-      <x:c r="C18" s="91"/>
+      <x:c r="C18" s="94"/>
       <x:c r="D18" s="45"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="45"/>
-      <x:c r="C19" s="91"/>
+      <x:c r="C19" s="94"/>
       <x:c r="D19" s="45"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="45"/>
-      <x:c r="C20" s="91"/>
+      <x:c r="C20" s="94"/>
       <x:c r="D20" s="45"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="45"/>
-      <x:c r="C21" s="91"/>
+      <x:c r="C21" s="94"/>
       <x:c r="D21" s="45"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="45"/>
-      <x:c r="C22" s="91"/>
+      <x:c r="C22" s="94"/>
       <x:c r="D22" s="45"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="45"/>
-      <x:c r="C23" s="91"/>
+      <x:c r="C23" s="94"/>
       <x:c r="D23" s="45"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="45"/>
-      <x:c r="C24" s="91"/>
+      <x:c r="C24" s="94"/>
       <x:c r="D24" s="45"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="45"/>
-      <x:c r="C25" s="91"/>
+      <x:c r="C25" s="94"/>
       <x:c r="D25" s="45"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="45"/>
-      <x:c r="C26" s="91"/>
+      <x:c r="C26" s="94"/>
       <x:c r="D26" s="45"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="45"/>
-      <x:c r="C27" s="91"/>
+      <x:c r="C27" s="94"/>
       <x:c r="D27" s="45"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="45"/>
-      <x:c r="C28" s="91"/>
+      <x:c r="C28" s="94"/>
       <x:c r="D28" s="45"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="45"/>
-      <x:c r="C29" s="91"/>
+      <x:c r="C29" s="94"/>
       <x:c r="D29" s="45"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="45"/>
-      <x:c r="C30" s="91"/>
+      <x:c r="C30" s="94"/>
       <x:c r="D30" s="45"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="45"/>
-      <x:c r="C31" s="91"/>
+      <x:c r="C31" s="94"/>
       <x:c r="D31" s="45"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="45"/>
-      <x:c r="C32" s="91"/>
+      <x:c r="C32" s="94"/>
       <x:c r="D32" s="45"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="45"/>
-      <x:c r="C33" s="91"/>
+      <x:c r="C33" s="94"/>
       <x:c r="D33" s="45"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="45"/>
-      <x:c r="C34" s="91"/>
+      <x:c r="C34" s="94"/>
       <x:c r="D34" s="45"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="45"/>
-      <x:c r="C35" s="91"/>
+      <x:c r="C35" s="94"/>
       <x:c r="D35" s="45"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="45"/>
-      <x:c r="C36" s="91"/>
+      <x:c r="C36" s="94"/>
       <x:c r="D36" s="45"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="45"/>
-      <x:c r="C37" s="91"/>
+      <x:c r="C37" s="94"/>
       <x:c r="D37" s="45"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="45"/>
-      <x:c r="C38" s="91"/>
+      <x:c r="C38" s="94"/>
       <x:c r="D38" s="45"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="45"/>
-      <x:c r="C39" s="91"/>
+      <x:c r="C39" s="94"/>
       <x:c r="D39" s="45"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="45"/>
-      <x:c r="C40" s="91"/>
+      <x:c r="C40" s="94"/>
       <x:c r="D40" s="45"/>
     </x:row>
   </x:sheetData>
@@ -2410,7 +2424,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94a2875ba50b48e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb072a427814a8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2430,300 +2444,300 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="69" t="str">
-        <x:v>Ambito scadenza</x:v>
-      </x:c>
-      <x:c r="B1" s="70" t="str">
-        <x:v>Username o targa o codice</x:v>
-      </x:c>
-      <x:c r="C1" s="70" t="str">
-        <x:v>Tipo scadenza</x:v>
-      </x:c>
-      <x:c r="D1" s="70" t="str">
-        <x:v>Data scadenza</x:v>
-      </x:c>
-      <x:c r="E1" s="70" t="str">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Ambito scadenza *</x:v>
+      </x:c>
+      <x:c r="B1" s="72" t="str">
+        <x:v>Username o targa o codice *</x:v>
+      </x:c>
+      <x:c r="C1" s="72" t="str">
+        <x:v>Tipo scadenza *</x:v>
+      </x:c>
+      <x:c r="D1" s="72" t="str">
+        <x:v>Data scadenza *</x:v>
+      </x:c>
+      <x:c r="E1" s="73" t="str">
         <x:v>Numero documento</x:v>
       </x:c>
-      <x:c r="F1" s="70" t="str">
+      <x:c r="F1" s="73" t="str">
         <x:v>Responsabile</x:v>
       </x:c>
-      <x:c r="G1" s="70" t="str">
+      <x:c r="G1" s="73" t="str">
         <x:v>Visibile in app</x:v>
       </x:c>
-      <x:c r="H1" s="71" t="str">
+      <x:c r="H1" s="74" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="72" t="str">
+      <x:c r="A2" s="75" t="str">
         <x:v>mezzo</x:v>
       </x:c>
-      <x:c r="B2" s="73" t="str">
+      <x:c r="B2" s="76" t="str">
         <x:v>AB123CD</x:v>
       </x:c>
-      <x:c r="C2" s="74" t="str">
+      <x:c r="C2" s="77" t="str">
         <x:v>Revisione mezzo</x:v>
       </x:c>
-      <x:c r="D2" s="89" t="str">
+      <x:c r="D2" s="92" t="str">
         <x:v>2026-12-15</x:v>
       </x:c>
-      <x:c r="E2" s="73" t="str">
+      <x:c r="E2" s="76" t="str">
         <x:v>REV-AB123CD</x:v>
       </x:c>
-      <x:c r="F2" s="74" t="str">
+      <x:c r="F2" s="77" t="str">
         <x:v>Ufficio flotta</x:v>
       </x:c>
-      <x:c r="G2" s="74" t="str">
+      <x:c r="G2" s="77" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="H2" s="75" t="str">
+      <x:c r="H2" s="78" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="72" t="str">
+      <x:c r="A3" s="75" t="str">
         <x:v>attrezzatura</x:v>
       </x:c>
-      <x:c r="B3" s="73" t="str">
+      <x:c r="B3" s="76" t="str">
         <x:v>MUL-01</x:v>
       </x:c>
-      <x:c r="C3" s="74" t="str">
+      <x:c r="C3" s="77" t="str">
         <x:v>Verifica sicurezza muletto</x:v>
       </x:c>
-      <x:c r="D3" s="89" t="str">
+      <x:c r="D3" s="92" t="str">
         <x:v>2026-10-10</x:v>
       </x:c>
-      <x:c r="E3" s="73" t="str">
+      <x:c r="E3" s="76" t="str">
         <x:v>CHK-MUL01</x:v>
       </x:c>
-      <x:c r="F3" s="74" t="str">
+      <x:c r="F3" s="77" t="str">
         <x:v>Responsabile magazzino</x:v>
       </x:c>
-      <x:c r="G3" s="74" t="str">
+      <x:c r="G3" s="77" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="H3" s="75" t="str"/>
+      <x:c r="H3" s="78" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="72" t="str">
+      <x:c r="A4" s="75" t="str">
         <x:v>persona</x:v>
       </x:c>
-      <x:c r="B4" s="73" t="str">
+      <x:c r="B4" s="76" t="str">
         <x:v>luca.neri</x:v>
       </x:c>
-      <x:c r="C4" s="74" t="str">
+      <x:c r="C4" s="77" t="str">
         <x:v>Visita medica</x:v>
       </x:c>
-      <x:c r="D4" s="89" t="str">
+      <x:c r="D4" s="92" t="str">
         <x:v>2027-02-01</x:v>
       </x:c>
-      <x:c r="E4" s="73" t="str">
+      <x:c r="E4" s="76" t="str">
         <x:v>VM-LUCA</x:v>
       </x:c>
-      <x:c r="F4" s="74" t="str">
+      <x:c r="F4" s="77" t="str">
         <x:v>Ufficio personale</x:v>
       </x:c>
-      <x:c r="G4" s="74" t="str">
+      <x:c r="G4" s="77" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="H4" s="75" t="str"/>
+      <x:c r="H4" s="78" t="str"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="76" t="str">
+      <x:c r="A5" s="79" t="str">
         <x:v>azienda</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str"/>
-      <x:c r="C5" s="78" t="str">
+      <x:c r="B5" s="80" t="str"/>
+      <x:c r="C5" s="81" t="str">
         <x:v>Polizza sede</x:v>
       </x:c>
-      <x:c r="D5" s="90" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>2027-01-31</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="80" t="str">
         <x:v>POL-SEDE</x:v>
       </x:c>
-      <x:c r="F5" s="78" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Amministrazione</x:v>
       </x:c>
-      <x:c r="G5" s="78" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="H5" s="79" t="str"/>
+      <x:c r="H5" s="82" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="B6" s="45"/>
-      <x:c r="D6" s="91"/>
+      <x:c r="D6" s="94"/>
       <x:c r="E6" s="45"/>
     </x:row>
     <x:row r="7">
       <x:c r="B7" s="45"/>
-      <x:c r="D7" s="91"/>
+      <x:c r="D7" s="94"/>
       <x:c r="E7" s="45"/>
     </x:row>
     <x:row r="8">
       <x:c r="B8" s="45"/>
-      <x:c r="D8" s="91"/>
+      <x:c r="D8" s="94"/>
       <x:c r="E8" s="45"/>
     </x:row>
     <x:row r="9">
       <x:c r="B9" s="45"/>
-      <x:c r="D9" s="91"/>
+      <x:c r="D9" s="94"/>
       <x:c r="E9" s="45"/>
     </x:row>
     <x:row r="10">
       <x:c r="B10" s="45"/>
-      <x:c r="D10" s="91"/>
+      <x:c r="D10" s="94"/>
       <x:c r="E10" s="45"/>
     </x:row>
     <x:row r="11">
       <x:c r="B11" s="45"/>
-      <x:c r="D11" s="91"/>
+      <x:c r="D11" s="94"/>
       <x:c r="E11" s="45"/>
     </x:row>
     <x:row r="12">
       <x:c r="B12" s="45"/>
-      <x:c r="D12" s="91"/>
+      <x:c r="D12" s="94"/>
       <x:c r="E12" s="45"/>
     </x:row>
     <x:row r="13">
       <x:c r="B13" s="45"/>
-      <x:c r="D13" s="91"/>
+      <x:c r="D13" s="94"/>
       <x:c r="E13" s="45"/>
     </x:row>
     <x:row r="14">
       <x:c r="B14" s="45"/>
-      <x:c r="D14" s="91"/>
+      <x:c r="D14" s="94"/>
       <x:c r="E14" s="45"/>
     </x:row>
     <x:row r="15">
       <x:c r="B15" s="45"/>
-      <x:c r="D15" s="91"/>
+      <x:c r="D15" s="94"/>
       <x:c r="E15" s="45"/>
     </x:row>
     <x:row r="16">
       <x:c r="B16" s="45"/>
-      <x:c r="D16" s="91"/>
+      <x:c r="D16" s="94"/>
       <x:c r="E16" s="45"/>
     </x:row>
     <x:row r="17">
       <x:c r="B17" s="45"/>
-      <x:c r="D17" s="91"/>
+      <x:c r="D17" s="94"/>
       <x:c r="E17" s="45"/>
     </x:row>
     <x:row r="18">
       <x:c r="B18" s="45"/>
-      <x:c r="D18" s="91"/>
+      <x:c r="D18" s="94"/>
       <x:c r="E18" s="45"/>
     </x:row>
     <x:row r="19">
       <x:c r="B19" s="45"/>
-      <x:c r="D19" s="91"/>
+      <x:c r="D19" s="94"/>
       <x:c r="E19" s="45"/>
     </x:row>
     <x:row r="20">
       <x:c r="B20" s="45"/>
-      <x:c r="D20" s="91"/>
+      <x:c r="D20" s="94"/>
       <x:c r="E20" s="45"/>
     </x:row>
     <x:row r="21">
       <x:c r="B21" s="45"/>
-      <x:c r="D21" s="91"/>
+      <x:c r="D21" s="94"/>
       <x:c r="E21" s="45"/>
     </x:row>
     <x:row r="22">
       <x:c r="B22" s="45"/>
-      <x:c r="D22" s="91"/>
+      <x:c r="D22" s="94"/>
       <x:c r="E22" s="45"/>
     </x:row>
     <x:row r="23">
       <x:c r="B23" s="45"/>
-      <x:c r="D23" s="91"/>
+      <x:c r="D23" s="94"/>
       <x:c r="E23" s="45"/>
     </x:row>
     <x:row r="24">
       <x:c r="B24" s="45"/>
-      <x:c r="D24" s="91"/>
+      <x:c r="D24" s="94"/>
       <x:c r="E24" s="45"/>
     </x:row>
     <x:row r="25">
       <x:c r="B25" s="45"/>
-      <x:c r="D25" s="91"/>
+      <x:c r="D25" s="94"/>
       <x:c r="E25" s="45"/>
     </x:row>
     <x:row r="26">
       <x:c r="B26" s="45"/>
-      <x:c r="D26" s="91"/>
+      <x:c r="D26" s="94"/>
       <x:c r="E26" s="45"/>
     </x:row>
     <x:row r="27">
       <x:c r="B27" s="45"/>
-      <x:c r="D27" s="91"/>
+      <x:c r="D27" s="94"/>
       <x:c r="E27" s="45"/>
     </x:row>
     <x:row r="28">
       <x:c r="B28" s="45"/>
-      <x:c r="D28" s="91"/>
+      <x:c r="D28" s="94"/>
       <x:c r="E28" s="45"/>
     </x:row>
     <x:row r="29">
       <x:c r="B29" s="45"/>
-      <x:c r="D29" s="91"/>
+      <x:c r="D29" s="94"/>
       <x:c r="E29" s="45"/>
     </x:row>
     <x:row r="30">
       <x:c r="B30" s="45"/>
-      <x:c r="D30" s="91"/>
+      <x:c r="D30" s="94"/>
       <x:c r="E30" s="45"/>
     </x:row>
     <x:row r="31">
       <x:c r="B31" s="45"/>
-      <x:c r="D31" s="91"/>
+      <x:c r="D31" s="94"/>
       <x:c r="E31" s="45"/>
     </x:row>
     <x:row r="32">
       <x:c r="B32" s="45"/>
-      <x:c r="D32" s="91"/>
+      <x:c r="D32" s="94"/>
       <x:c r="E32" s="45"/>
     </x:row>
     <x:row r="33">
       <x:c r="B33" s="45"/>
-      <x:c r="D33" s="91"/>
+      <x:c r="D33" s="94"/>
       <x:c r="E33" s="45"/>
     </x:row>
     <x:row r="34">
       <x:c r="B34" s="45"/>
-      <x:c r="D34" s="91"/>
+      <x:c r="D34" s="94"/>
       <x:c r="E34" s="45"/>
     </x:row>
     <x:row r="35">
       <x:c r="B35" s="45"/>
-      <x:c r="D35" s="91"/>
+      <x:c r="D35" s="94"/>
       <x:c r="E35" s="45"/>
     </x:row>
     <x:row r="36">
       <x:c r="B36" s="45"/>
-      <x:c r="D36" s="91"/>
+      <x:c r="D36" s="94"/>
       <x:c r="E36" s="45"/>
     </x:row>
     <x:row r="37">
       <x:c r="B37" s="45"/>
-      <x:c r="D37" s="91"/>
+      <x:c r="D37" s="94"/>
       <x:c r="E37" s="45"/>
     </x:row>
     <x:row r="38">
       <x:c r="B38" s="45"/>
-      <x:c r="D38" s="91"/>
+      <x:c r="D38" s="94"/>
       <x:c r="E38" s="45"/>
     </x:row>
     <x:row r="39">
       <x:c r="B39" s="45"/>
-      <x:c r="D39" s="91"/>
+      <x:c r="D39" s="94"/>
       <x:c r="E39" s="45"/>
     </x:row>
     <x:row r="40">
       <x:c r="B40" s="45"/>
-      <x:c r="D40" s="91"/>
+      <x:c r="D40" s="94"/>
       <x:c r="E40" s="45"/>
     </x:row>
   </x:sheetData>
@@ -2737,7 +2751,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7762e25b04804847"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recd29253bf854e25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Nasconde email tecnica accesso autisti
</commit_message>
<xml_diff>
--- a/public/templates/vygo-import-anagrafiche.xlsx
+++ b/public/templates/vygo-import-anagrafiche.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGGIMI" sheetId="1" r:id="R1b9db92d875c42db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autisti" sheetId="2" r:id="R3f85fe4ee0ba4457"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone" sheetId="3" r:id="Ra4dd991a72c24f85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mezzi" sheetId="4" r:id="Raea6b97d78374910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrezzature" sheetId="5" r:id="Rdafaa965b6e443db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenti autisti" sheetId="6" r:id="Rab9ad5692029472a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scadenze" sheetId="7" r:id="Rdeacfb7c719c499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGGIMI" sheetId="1" r:id="R6b97cc26e9ba45d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autisti" sheetId="2" r:id="R475cdd025e434ef4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone" sheetId="3" r:id="R0c33fa0c77cb417e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mezzi" sheetId="4" r:id="Rbd7499e515c24a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrezzature" sheetId="5" r:id="R5e92e58f960c46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenti autisti" sheetId="6" r:id="Rebf2be2ae2694766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scadenze" sheetId="7" r:id="R38a23e003ab94317"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -425,21 +425,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VygoAutisti" displayName="VygoAutisti" ref="A1:L12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:L12"/>
-  <x:tableColumns count="12">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VygoAutisti" displayName="VygoAutisti" ref="A1:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:K12"/>
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="Nome e cognome *"/>
     <x:tableColumn id="2" name="Username *"/>
     <x:tableColumn id="3" name="Password *"/>
     <x:tableColumn id="4" name="Telefono *"/>
-    <x:tableColumn id="5" name="Email"/>
-    <x:tableColumn id="6" name="Ruolo"/>
-    <x:tableColumn id="7" name="Deposito / sede"/>
-    <x:tableColumn id="8" name="Documento iniziale"/>
-    <x:tableColumn id="9" name="Scadenza documento"/>
-    <x:tableColumn id="10" name="Numero documento"/>
-    <x:tableColumn id="11" name="Visibile in app"/>
-    <x:tableColumn id="12" name="Note"/>
+    <x:tableColumn id="5" name="Ruolo"/>
+    <x:tableColumn id="6" name="Deposito / sede"/>
+    <x:tableColumn id="7" name="Documento iniziale"/>
+    <x:tableColumn id="8" name="Scadenza documento"/>
+    <x:tableColumn id="9" name="Numero documento"/>
+    <x:tableColumn id="10" name="Visibile in app"/>
+    <x:tableColumn id="11" name="Note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -883,14 +882,13 @@
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -907,27 +905,24 @@
         <x:v>Telefono *</x:v>
       </x:c>
       <x:c r="E1" s="73" t="str">
-        <x:v>Email</x:v>
+        <x:v>Ruolo</x:v>
       </x:c>
       <x:c r="F1" s="73" t="str">
-        <x:v>Ruolo</x:v>
+        <x:v>Deposito / sede</x:v>
       </x:c>
       <x:c r="G1" s="73" t="str">
-        <x:v>Deposito / sede</x:v>
+        <x:v>Documento iniziale</x:v>
       </x:c>
       <x:c r="H1" s="73" t="str">
-        <x:v>Documento iniziale</x:v>
+        <x:v>Scadenza documento</x:v>
       </x:c>
       <x:c r="I1" s="73" t="str">
-        <x:v>Scadenza documento</x:v>
+        <x:v>Numero documento</x:v>
       </x:c>
       <x:c r="J1" s="73" t="str">
-        <x:v>Numero documento</x:v>
-      </x:c>
-      <x:c r="K1" s="73" t="str">
         <x:v>Visibile in app</x:v>
       </x:c>
-      <x:c r="L1" s="74" t="str">
+      <x:c r="K1" s="74" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
@@ -945,27 +940,24 @@
         <x:v>+39 333 111 1111</x:v>
       </x:c>
       <x:c r="E2" s="77" t="str">
-        <x:v>mario.rossi@azienda.it</x:v>
+        <x:v>Autista bilico</x:v>
       </x:c>
       <x:c r="F2" s="77" t="str">
-        <x:v>Autista bilico</x:v>
+        <x:v>Verona</x:v>
       </x:c>
       <x:c r="G2" s="77" t="str">
-        <x:v>Verona</x:v>
+        <x:v>Patente C+E</x:v>
       </x:c>
       <x:c r="H2" s="77" t="str">
-        <x:v>Patente C+E</x:v>
+        <x:v>2027-05-31</x:v>
       </x:c>
       <x:c r="I2" s="92" t="str">
-        <x:v>2027-05-31</x:v>
+        <x:v>PCE12345</x:v>
       </x:c>
       <x:c r="J2" s="76" t="str">
-        <x:v>PCE12345</x:v>
-      </x:c>
-      <x:c r="K2" s="77" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="L2" s="78" t="str">
+      <x:c r="K2" s="78" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
@@ -983,27 +975,24 @@
         <x:v>+39 333 222 2222</x:v>
       </x:c>
       <x:c r="E3" s="81" t="str">
-        <x:v>anna.verdi@azienda.it</x:v>
+        <x:v>Autista furgone</x:v>
       </x:c>
       <x:c r="F3" s="81" t="str">
-        <x:v>Autista furgone</x:v>
+        <x:v>Milano</x:v>
       </x:c>
       <x:c r="G3" s="81" t="str">
-        <x:v>Milano</x:v>
+        <x:v>CQC</x:v>
       </x:c>
       <x:c r="H3" s="81" t="str">
-        <x:v>CQC</x:v>
+        <x:v>2027-11-30</x:v>
       </x:c>
       <x:c r="I3" s="93" t="str">
-        <x:v>2027-11-30</x:v>
+        <x:v>CQC9988</x:v>
       </x:c>
       <x:c r="J3" s="80" t="str">
-        <x:v>CQC9988</x:v>
-      </x:c>
-      <x:c r="K3" s="81" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="L3" s="82" t="str"/>
+      <x:c r="K3" s="82" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="B4" s="45"/>
@@ -1266,13 +1255,13 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="K2:K40">
+    <x:dataValidation type="list" sqref="J2:J40">
       <x:formula1>"si,no"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83883da298bc4138"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83ecd371c6a14f08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1583,7 +1572,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R271d9229258d40ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfe4ae7da9064f99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1841,7 +1830,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43c5a6c3ef8a47d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb48f3ac12b314391"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2146,7 +2135,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R762e134555874c91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb5cd81d802b4400"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2424,7 +2413,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb072a427814a8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R217f75393eb0412d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2751,7 +2740,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recd29253bf854e25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfa97270ca0a43c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Migliora guida Excel import Vygo
</commit_message>
<xml_diff>
--- a/public/templates/vygo-import-anagrafiche.xlsx
+++ b/public/templates/vygo-import-anagrafiche.xlsx
@@ -2,13 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGGIMI" sheetId="1" r:id="R6b97cc26e9ba45d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autisti" sheetId="2" r:id="R475cdd025e434ef4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone" sheetId="3" r:id="R0c33fa0c77cb417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mezzi" sheetId="4" r:id="Rbd7499e515c24a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrezzature" sheetId="5" r:id="R5e92e58f960c46b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenti autisti" sheetId="6" r:id="Rebf2be2ae2694766"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scadenze" sheetId="7" r:id="R38a23e003ab94317"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGGIMI" sheetId="1" r:id="Rf0a77dfa02274c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guida compilazione" sheetId="2" r:id="Rf886af51e7e6447f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzioni" sheetId="3" r:id="Rf996499bc92340d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autisti" sheetId="4" r:id="Raa2fb75d0ee34621"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone" sheetId="5" r:id="R83a33b0413a84115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mezzi" sheetId="6" r:id="R422a72ab54f8400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrezzature" sheetId="7" r:id="Ra6dbd29f7962403d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenti autisti" sheetId="8" r:id="R129c9c3bd1cb4587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scadenze" sheetId="9" r:id="R92c0b8667ecb4d55"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -189,7 +191,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="95">
+  <x:cellXfs count="97">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -295,7 +297,6 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -306,13 +307,7 @@
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -322,71 +317,84 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -425,7 +433,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VygoAutisti" displayName="VygoAutisti" ref="A1:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VygoGuidaCompilazione" displayName="VygoGuidaCompilazione" ref="A1:D22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:D22"/>
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="Area / campo"/>
+    <x:tableColumn id="2" name="Come scriverlo"/>
+    <x:tableColumn id="3" name="Esempi corretti"/>
+    <x:tableColumn id="4" name="Da evitare"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="VygoOpzioniImport" displayName="VygoOpzioniImport" ref="A1:E47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:E47"/>
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Foglio"/>
+    <x:tableColumn id="2" name="Campo"/>
+    <x:tableColumn id="3" name="Scrivi così"/>
+    <x:tableColumn id="4" name="Altri esempi accettati"/>
+    <x:tableColumn id="5" name="Quando usarlo"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VygoAutisti" displayName="VygoAutisti" ref="A1:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:K12"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Nome e cognome *"/>
@@ -444,8 +479,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="VygoPersone" displayName="VygoPersone" ref="A1:J12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="VygoPersone" displayName="VygoPersone" ref="A1:J12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:J12"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Nome e cognome *"/>
@@ -463,8 +498,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VygoMezzi" displayName="VygoMezzi" ref="A1:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="VygoMezzi" displayName="VygoMezzi" ref="A1:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G12"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Targa *"/>
@@ -479,8 +514,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="VygoAttrezzature" displayName="VygoAttrezzature" ref="A1:F12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="VygoAttrezzature" displayName="VygoAttrezzature" ref="A1:F12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:F12"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Codice *"/>
@@ -494,8 +529,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="VygoDocumentiAutisti" displayName="VygoDocumentiAutisti" ref="A1:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="VygoDocumentiAutisti" displayName="VygoDocumentiAutisti" ref="A1:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G12"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Username autista *"/>
@@ -510,8 +545,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="VygoScadenze" displayName="VygoScadenze" ref="A1:H12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="VygoScadenze" displayName="VygoScadenze" ref="A1:H12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:H12"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Ambito scadenza *"/>
@@ -878,6 +913,885 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="64" t="str">
+        <x:v>Area / campo</x:v>
+      </x:c>
+      <x:c r="B1" s="65" t="str">
+        <x:v>Come scriverlo</x:v>
+      </x:c>
+      <x:c r="C1" s="65" t="str">
+        <x:v>Esempi corretti</x:v>
+      </x:c>
+      <x:c r="D1" s="66" t="str">
+        <x:v>Da evitare</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="67" t="str">
+        <x:v>Regola generale</x:v>
+      </x:c>
+      <x:c r="B2" s="68" t="str">
+        <x:v>Non cambiare mai i titoli delle colonne. Vygo li usa per capire cosa importare.</x:v>
+      </x:c>
+      <x:c r="C2" s="68" t="str">
+        <x:v>Compila le righe sotto ai titoli e cancella solo le righe esempio.</x:v>
+      </x:c>
+      <x:c r="D2" s="69" t="str">
+        <x:v>Non rinominare fogli o colonne.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="67" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B3" s="68" t="str">
+        <x:v>Usa sempre AAAA-MM-GG quando puoi.</x:v>
+      </x:c>
+      <x:c r="C3" s="68" t="str">
+        <x:v>2027-05-31, 2026-12-15</x:v>
+      </x:c>
+      <x:c r="D3" s="69" t="str">
+        <x:v>Evita testi come "fine mese" o "tra un anno".</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="67" t="str">
+        <x:v>Username</x:v>
+      </x:c>
+      <x:c r="B4" s="68" t="str">
+        <x:v>Scrivi nomi semplici, minuscoli, senza spazi.</x:v>
+      </x:c>
+      <x:c r="C4" s="68" t="str">
+        <x:v>mario.rossi, paola.ufficio, magazzino1</x:v>
+      </x:c>
+      <x:c r="D4" s="69" t="str">
+        <x:v>Evita accenti, apostrofi, spazi e caratteri strani.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="67" t="str">
+        <x:v>Password</x:v>
+      </x:c>
+      <x:c r="B5" s="68" t="str">
+        <x:v>Minimo 8 caratteri. Deve essere quella che poi comunichi alla persona.</x:v>
+      </x:c>
+      <x:c r="C5" s="68" t="str">
+        <x:v>Vygo2026!, Spedi2026</x:v>
+      </x:c>
+      <x:c r="D5" s="69" t="str">
+        <x:v>Non lasciare vuota la password per utenti che devono entrare in app.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="67" t="str">
+        <x:v>Telefono</x:v>
+      </x:c>
+      <x:c r="B6" s="68" t="str">
+        <x:v>Meglio con prefisso internazionale.</x:v>
+      </x:c>
+      <x:c r="C6" s="68" t="str">
+        <x:v>+39 333 111 1111</x:v>
+      </x:c>
+      <x:c r="D6" s="69" t="str">
+        <x:v>Evita numeri senza prefisso se l azienda lavora anche fuori Italia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="67" t="str">
+        <x:v>Mezzi - Categoria mezzo</x:v>
+      </x:c>
+      <x:c r="B7" s="68" t="str">
+        <x:v>Usa una di queste parole: furgone, motrice, trattore, semirimorchio.</x:v>
+      </x:c>
+      <x:c r="C7" s="68" t="str">
+        <x:v>trattore per il trattore stradale; semirimorchio per il rimorchio agganciato.</x:v>
+      </x:c>
+      <x:c r="D7" s="69" t="str">
+        <x:v>Non scrivere l allestimento nella categoria mezzo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="67" t="str">
+        <x:v>Mezzi - Allestimento</x:v>
+      </x:c>
+      <x:c r="B8" s="68" t="str">
+        <x:v>Qui puoi descrivere il mezzo liberamente.</x:v>
+      </x:c>
+      <x:c r="C8" s="68" t="str">
+        <x:v>centinato, cassonato, frigo, isotermico, telonato, pianale, ribaltabile, cisterna, portacontainer, sponda idraulica</x:v>
+      </x:c>
+      <x:c r="D8" s="69" t="str">
+        <x:v>Non usare l allestimento al posto della categoria mezzo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="67" t="str">
+        <x:v>Attrezzature</x:v>
+      </x:c>
+      <x:c r="B9" s="68" t="str">
+        <x:v>Usa una di queste parole: muletto, transpallet, attrezzatura, altro.</x:v>
+      </x:c>
+      <x:c r="C9" s="68" t="str">
+        <x:v>muletto per carrello elevatore; transpallet per transpallet elettrico/manuale.</x:v>
+      </x:c>
+      <x:c r="D9" s="69" t="str">
+        <x:v>Forche, batterie e caricabatterie possono stare in modello/note se non sono mezzi autonomi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="67" t="str">
+        <x:v>Persone - Reparto</x:v>
+      </x:c>
+      <x:c r="B10" s="68" t="str">
+        <x:v>Usa ufficio o magazzino.</x:v>
+      </x:c>
+      <x:c r="C10" s="68" t="str">
+        <x:v>ufficio per traffico/amministrazione; magazzino per carrellisti e operatori magazzino.</x:v>
+      </x:c>
+      <x:c r="D10" s="69" t="str">
+        <x:v>Non usare "autisti" nel foglio Persone: gli autisti hanno il loro foglio.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="67" t="str">
+        <x:v>Persone - Ruolo</x:v>
+      </x:c>
+      <x:c r="B11" s="68" t="str">
+        <x:v>Usa ruoli chiari e coerenti.</x:v>
+      </x:c>
+      <x:c r="C11" s="68" t="str">
+        <x:v>Impiegato ufficio, Manager, Magazziniere, Carrellista</x:v>
+      </x:c>
+      <x:c r="D11" s="69" t="str">
+        <x:v>La mansione dettagliata va nella colonna Mansione.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B12" s="68" t="str">
+        <x:v>Scrivi il tipo documento come vuoi vederlo in Vygo.</x:v>
+      </x:c>
+      <x:c r="C12" s="68" t="str">
+        <x:v>Patente B, Patente C, Patente C+E, CQC merci, Carta tachigrafica, Visita medica, ADR base, ADR cisterna</x:v>
+      </x:c>
+      <x:c r="D12" s="69" t="str">
+        <x:v>Non mettere documenti del muletto qui: quelli vanno in Scadenze con ambito attrezzatura.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="67" t="str">
+        <x:v>Scadenze - Ambito</x:v>
+      </x:c>
+      <x:c r="B13" s="68" t="str">
+        <x:v>Usa autista, persona, mezzo, attrezzatura o azienda.</x:v>
+      </x:c>
+      <x:c r="C13" s="68" t="str">
+        <x:v>mezzo + AB123CD per revisione; persona + luca.neri per visita medica; attrezzatura + MUL-01 per verifica muletto.</x:v>
+      </x:c>
+      <x:c r="D13" s="69" t="str">
+        <x:v>Se ambito e target non combaciano, Vygo segnala errore in anteprima.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="67" t="str">
+        <x:v>Scadenze - Target</x:v>
+      </x:c>
+      <x:c r="B14" s="68" t="str">
+        <x:v>Per autista/persona usa username. Per mezzo usa targa. Per attrezzatura usa codice.</x:v>
+      </x:c>
+      <x:c r="C14" s="68" t="str">
+        <x:v>mario.rossi, AB123CD, MUL-01</x:v>
+      </x:c>
+      <x:c r="D14" s="69" t="str">
+        <x:v>Per scadenza azienda il target puo restare vuoto.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="70" t="str">
+        <x:v>Visibile in app</x:v>
+      </x:c>
+      <x:c r="B15" s="71" t="str">
+        <x:v>Scrivi si se l utente deve vedere il documento o la scadenza nella sua app. Scrivi no se resta solo aziendale.</x:v>
+      </x:c>
+      <x:c r="C15" s="71" t="str">
+        <x:v>si, no</x:v>
+      </x:c>
+      <x:c r="D15" s="72" t="str">
+        <x:v>Non usare forse, ok, x o altri valori.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22a8c0763c5e4a35"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="64" t="str">
+        <x:v>Foglio</x:v>
+      </x:c>
+      <x:c r="B1" s="65" t="str">
+        <x:v>Campo</x:v>
+      </x:c>
+      <x:c r="C1" s="65" t="str">
+        <x:v>Scrivi così</x:v>
+      </x:c>
+      <x:c r="D1" s="65" t="str">
+        <x:v>Altri esempi accettati</x:v>
+      </x:c>
+      <x:c r="E1" s="66" t="str">
+        <x:v>Quando usarlo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B2" s="68" t="str">
+        <x:v>Categoria mezzo</x:v>
+      </x:c>
+      <x:c r="C2" s="68" t="str">
+        <x:v>furgone</x:v>
+      </x:c>
+      <x:c r="D2" s="68" t="str">
+        <x:v>van</x:v>
+      </x:c>
+      <x:c r="E2" s="69" t="str">
+        <x:v>Furgoni e veicoli leggeri</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B3" s="68" t="str">
+        <x:v>Categoria mezzo</x:v>
+      </x:c>
+      <x:c r="C3" s="68" t="str">
+        <x:v>motrice</x:v>
+      </x:c>
+      <x:c r="D3" s="68" t="str"/>
+      <x:c r="E3" s="69" t="str">
+        <x:v>Motrice rigida</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B4" s="68" t="str">
+        <x:v>Categoria mezzo</x:v>
+      </x:c>
+      <x:c r="C4" s="68" t="str">
+        <x:v>trattore</x:v>
+      </x:c>
+      <x:c r="D4" s="68" t="str">
+        <x:v>bilico</x:v>
+      </x:c>
+      <x:c r="E4" s="69" t="str">
+        <x:v>Trattore stradale che aggancia semirimorchio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B5" s="68" t="str">
+        <x:v>Categoria mezzo</x:v>
+      </x:c>
+      <x:c r="C5" s="68" t="str">
+        <x:v>semirimorchio</x:v>
+      </x:c>
+      <x:c r="D5" s="68" t="str">
+        <x:v>semi</x:v>
+      </x:c>
+      <x:c r="E5" s="69" t="str">
+        <x:v>Semirimorchio agganciabile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B6" s="68" t="str">
+        <x:v>Allestimento</x:v>
+      </x:c>
+      <x:c r="C6" s="68" t="str">
+        <x:v>centinato</x:v>
+      </x:c>
+      <x:c r="D6" s="68" t="str"/>
+      <x:c r="E6" s="69" t="str">
+        <x:v>Descrizione libera del mezzo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B7" s="68" t="str">
+        <x:v>Allestimento</x:v>
+      </x:c>
+      <x:c r="C7" s="68" t="str">
+        <x:v>cassonato</x:v>
+      </x:c>
+      <x:c r="D7" s="68" t="str"/>
+      <x:c r="E7" s="69" t="str">
+        <x:v>Descrizione libera del mezzo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B8" s="68" t="str">
+        <x:v>Allestimento</x:v>
+      </x:c>
+      <x:c r="C8" s="68" t="str">
+        <x:v>frigo / isotermico</x:v>
+      </x:c>
+      <x:c r="D8" s="68" t="str"/>
+      <x:c r="E8" s="69" t="str">
+        <x:v>Descrizione libera del mezzo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="67" t="str">
+        <x:v>Mezzi</x:v>
+      </x:c>
+      <x:c r="B9" s="68" t="str">
+        <x:v>Allestimento</x:v>
+      </x:c>
+      <x:c r="C9" s="68" t="str">
+        <x:v>telonato / pianale / ribaltabile</x:v>
+      </x:c>
+      <x:c r="D9" s="68" t="str"/>
+      <x:c r="E9" s="69" t="str">
+        <x:v>Descrizione libera del mezzo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="67" t="str">
+        <x:v>Attrezzature</x:v>
+      </x:c>
+      <x:c r="B10" s="68" t="str">
+        <x:v>Tipo attrezzatura</x:v>
+      </x:c>
+      <x:c r="C10" s="68" t="str">
+        <x:v>muletto</x:v>
+      </x:c>
+      <x:c r="D10" s="68" t="str">
+        <x:v>forklift</x:v>
+      </x:c>
+      <x:c r="E10" s="69" t="str">
+        <x:v>Carrello elevatore</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="67" t="str">
+        <x:v>Attrezzature</x:v>
+      </x:c>
+      <x:c r="B11" s="68" t="str">
+        <x:v>Tipo attrezzatura</x:v>
+      </x:c>
+      <x:c r="C11" s="68" t="str">
+        <x:v>transpallet</x:v>
+      </x:c>
+      <x:c r="D11" s="68" t="str">
+        <x:v>pallet</x:v>
+      </x:c>
+      <x:c r="E11" s="69" t="str">
+        <x:v>Transpallet manuale o elettrico</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="67" t="str">
+        <x:v>Attrezzature</x:v>
+      </x:c>
+      <x:c r="B12" s="68" t="str">
+        <x:v>Tipo attrezzatura</x:v>
+      </x:c>
+      <x:c r="C12" s="68" t="str">
+        <x:v>attrezzatura</x:v>
+      </x:c>
+      <x:c r="D12" s="68" t="str"/>
+      <x:c r="E12" s="69" t="str">
+        <x:v>Altra attrezzatura di magazzino</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="67" t="str">
+        <x:v>Attrezzature</x:v>
+      </x:c>
+      <x:c r="B13" s="68" t="str">
+        <x:v>Tipo attrezzatura</x:v>
+      </x:c>
+      <x:c r="C13" s="68" t="str">
+        <x:v>altro</x:v>
+      </x:c>
+      <x:c r="D13" s="68" t="str"/>
+      <x:c r="E13" s="69" t="str">
+        <x:v>Quando non rientra nelle voci precedenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="67" t="str">
+        <x:v>Persone</x:v>
+      </x:c>
+      <x:c r="B14" s="68" t="str">
+        <x:v>Reparto</x:v>
+      </x:c>
+      <x:c r="C14" s="68" t="str">
+        <x:v>ufficio</x:v>
+      </x:c>
+      <x:c r="D14" s="68" t="str"/>
+      <x:c r="E14" s="69" t="str">
+        <x:v>Traffico, amministrazione, direzione, operativo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="67" t="str">
+        <x:v>Persone</x:v>
+      </x:c>
+      <x:c r="B15" s="68" t="str">
+        <x:v>Reparto</x:v>
+      </x:c>
+      <x:c r="C15" s="68" t="str">
+        <x:v>magazzino</x:v>
+      </x:c>
+      <x:c r="D15" s="68" t="str"/>
+      <x:c r="E15" s="69" t="str">
+        <x:v>Magazzino e carrellisti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="67" t="str">
+        <x:v>Persone</x:v>
+      </x:c>
+      <x:c r="B16" s="68" t="str">
+        <x:v>Ruolo</x:v>
+      </x:c>
+      <x:c r="C16" s="68" t="str">
+        <x:v>Impiegato ufficio</x:v>
+      </x:c>
+      <x:c r="D16" s="68" t="str">
+        <x:v>impiegato, office</x:v>
+      </x:c>
+      <x:c r="E16" s="69" t="str">
+        <x:v>Ufficio traffico/amministrazione</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="67" t="str">
+        <x:v>Persone</x:v>
+      </x:c>
+      <x:c r="B17" s="68" t="str">
+        <x:v>Ruolo</x:v>
+      </x:c>
+      <x:c r="C17" s="68" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D17" s="68" t="str">
+        <x:v>responsabile</x:v>
+      </x:c>
+      <x:c r="E17" s="69" t="str">
+        <x:v>Responsabile o titolare operativo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="67" t="str">
+        <x:v>Persone</x:v>
+      </x:c>
+      <x:c r="B18" s="68" t="str">
+        <x:v>Ruolo</x:v>
+      </x:c>
+      <x:c r="C18" s="68" t="str">
+        <x:v>Magazziniere</x:v>
+      </x:c>
+      <x:c r="D18" s="68" t="str">
+        <x:v>warehouse</x:v>
+      </x:c>
+      <x:c r="E18" s="69" t="str">
+        <x:v>Operatore magazzino</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="67" t="str">
+        <x:v>Persone</x:v>
+      </x:c>
+      <x:c r="B19" s="68" t="str">
+        <x:v>Ruolo</x:v>
+      </x:c>
+      <x:c r="C19" s="68" t="str">
+        <x:v>Carrellista</x:v>
+      </x:c>
+      <x:c r="D19" s="68" t="str">
+        <x:v>forklift</x:v>
+      </x:c>
+      <x:c r="E19" s="69" t="str">
+        <x:v>Operatore muletto/carrello</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B20" s="68" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="C20" s="68" t="str">
+        <x:v>Patente B</x:v>
+      </x:c>
+      <x:c r="D20" s="68" t="str"/>
+      <x:c r="E20" s="69" t="str">
+        <x:v>Documento autista</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B21" s="68" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="C21" s="68" t="str">
+        <x:v>Patente C</x:v>
+      </x:c>
+      <x:c r="D21" s="68" t="str"/>
+      <x:c r="E21" s="69" t="str">
+        <x:v>Documento autista</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B22" s="68" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="C22" s="68" t="str">
+        <x:v>Patente C+E</x:v>
+      </x:c>
+      <x:c r="D22" s="68" t="str"/>
+      <x:c r="E22" s="69" t="str">
+        <x:v>Documento autista</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B23" s="68" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="C23" s="68" t="str">
+        <x:v>CQC merci</x:v>
+      </x:c>
+      <x:c r="D23" s="68" t="str">
+        <x:v>CQC</x:v>
+      </x:c>
+      <x:c r="E23" s="69" t="str">
+        <x:v>Documento autista</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B24" s="68" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="C24" s="68" t="str">
+        <x:v>Carta tachigrafica</x:v>
+      </x:c>
+      <x:c r="D24" s="68" t="str"/>
+      <x:c r="E24" s="69" t="str">
+        <x:v>Documento autista</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B25" s="68" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="C25" s="68" t="str">
+        <x:v>Visita medica</x:v>
+      </x:c>
+      <x:c r="D25" s="68" t="str"/>
+      <x:c r="E25" s="69" t="str">
+        <x:v>Scadenza sanitaria</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="67" t="str">
+        <x:v>Documenti autisti</x:v>
+      </x:c>
+      <x:c r="B26" s="68" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="C26" s="68" t="str">
+        <x:v>ADR base / ADR cisterna</x:v>
+      </x:c>
+      <x:c r="D26" s="68" t="str"/>
+      <x:c r="E26" s="69" t="str">
+        <x:v>Abilitazione merci pericolose</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B27" s="68" t="str">
+        <x:v>Ambito scadenza</x:v>
+      </x:c>
+      <x:c r="C27" s="68" t="str">
+        <x:v>autista</x:v>
+      </x:c>
+      <x:c r="D27" s="68" t="str">
+        <x:v>driver</x:v>
+      </x:c>
+      <x:c r="E27" s="69" t="str">
+        <x:v>Usa username autista come target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B28" s="68" t="str">
+        <x:v>Ambito scadenza</x:v>
+      </x:c>
+      <x:c r="C28" s="68" t="str">
+        <x:v>persona</x:v>
+      </x:c>
+      <x:c r="D28" s="68" t="str">
+        <x:v>dipendente</x:v>
+      </x:c>
+      <x:c r="E28" s="69" t="str">
+        <x:v>Usa username persona come target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B29" s="68" t="str">
+        <x:v>Ambito scadenza</x:v>
+      </x:c>
+      <x:c r="C29" s="68" t="str">
+        <x:v>mezzo</x:v>
+      </x:c>
+      <x:c r="D29" s="68" t="str">
+        <x:v>targa, flotta</x:v>
+      </x:c>
+      <x:c r="E29" s="69" t="str">
+        <x:v>Usa targa come target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B30" s="68" t="str">
+        <x:v>Ambito scadenza</x:v>
+      </x:c>
+      <x:c r="C30" s="68" t="str">
+        <x:v>attrezzatura</x:v>
+      </x:c>
+      <x:c r="D30" s="68" t="str">
+        <x:v>muletto</x:v>
+      </x:c>
+      <x:c r="E30" s="69" t="str">
+        <x:v>Usa codice attrezzatura come target</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B31" s="68" t="str">
+        <x:v>Ambito scadenza</x:v>
+      </x:c>
+      <x:c r="C31" s="68" t="str">
+        <x:v>azienda</x:v>
+      </x:c>
+      <x:c r="D31" s="68" t="str">
+        <x:v>company</x:v>
+      </x:c>
+      <x:c r="E31" s="69" t="str">
+        <x:v>Target vuoto</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B32" s="68" t="str">
+        <x:v>Tipo scadenza mezzo</x:v>
+      </x:c>
+      <x:c r="C32" s="68" t="str">
+        <x:v>Revisione mezzo</x:v>
+      </x:c>
+      <x:c r="D32" s="68" t="str"/>
+      <x:c r="E32" s="69" t="str">
+        <x:v>Scadenza flotta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B33" s="68" t="str">
+        <x:v>Tipo scadenza mezzo</x:v>
+      </x:c>
+      <x:c r="C33" s="68" t="str">
+        <x:v>Assicurazione</x:v>
+      </x:c>
+      <x:c r="D33" s="68" t="str"/>
+      <x:c r="E33" s="69" t="str">
+        <x:v>Scadenza flotta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B34" s="68" t="str">
+        <x:v>Tipo scadenza mezzo</x:v>
+      </x:c>
+      <x:c r="C34" s="68" t="str">
+        <x:v>Bollo</x:v>
+      </x:c>
+      <x:c r="D34" s="68" t="str"/>
+      <x:c r="E34" s="69" t="str">
+        <x:v>Scadenza flotta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B35" s="68" t="str">
+        <x:v>Tipo scadenza mezzo</x:v>
+      </x:c>
+      <x:c r="C35" s="68" t="str">
+        <x:v>Manutenzione programmata</x:v>
+      </x:c>
+      <x:c r="D35" s="68" t="str"/>
+      <x:c r="E35" s="69" t="str">
+        <x:v>Scadenza flotta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B36" s="68" t="str">
+        <x:v>Tipo scadenza attrezzatura</x:v>
+      </x:c>
+      <x:c r="C36" s="68" t="str">
+        <x:v>Verifica sicurezza muletto</x:v>
+      </x:c>
+      <x:c r="D36" s="68" t="str"/>
+      <x:c r="E36" s="69" t="str">
+        <x:v>Scadenza magazzino</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B37" s="68" t="str">
+        <x:v>Tipo scadenza attrezzatura</x:v>
+      </x:c>
+      <x:c r="C37" s="68" t="str">
+        <x:v>Manutenzione muletto</x:v>
+      </x:c>
+      <x:c r="D37" s="68" t="str"/>
+      <x:c r="E37" s="69" t="str">
+        <x:v>Scadenza magazzino</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="67" t="str">
+        <x:v>Scadenze</x:v>
+      </x:c>
+      <x:c r="B38" s="68" t="str">
+        <x:v>Tipo scadenza persona</x:v>
+      </x:c>
+      <x:c r="C38" s="68" t="str">
+        <x:v>Visita medica</x:v>
+      </x:c>
+      <x:c r="D38" s="68" t="str"/>
+      <x:c r="E38" s="69" t="str">
+        <x:v>Scadenza persona</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="67" t="str">
+        <x:v>Valori comuni</x:v>
+      </x:c>
+      <x:c r="B39" s="68" t="str">
+        <x:v>Visibile in app</x:v>
+      </x:c>
+      <x:c r="C39" s="68" t="str">
+        <x:v>si</x:v>
+      </x:c>
+      <x:c r="D39" s="68" t="str"/>
+      <x:c r="E39" s="69" t="str">
+        <x:v>L utente lo vede nella sua app</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="70" t="str">
+        <x:v>Valori comuni</x:v>
+      </x:c>
+      <x:c r="B40" s="71" t="str">
+        <x:v>Visibile in app</x:v>
+      </x:c>
+      <x:c r="C40" s="71" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D40" s="71" t="str"/>
+      <x:c r="E40" s="72" t="str">
+        <x:v>Resta solo nella dashboard azienda</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b8d1b7341f541e2"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
@@ -892,366 +1806,366 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="71" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Nome e cognome *</x:v>
       </x:c>
-      <x:c r="B1" s="72" t="str">
+      <x:c r="B1" s="82" t="str">
         <x:v>Username *</x:v>
       </x:c>
-      <x:c r="C1" s="72" t="str">
+      <x:c r="C1" s="82" t="str">
         <x:v>Password *</x:v>
       </x:c>
-      <x:c r="D1" s="72" t="str">
+      <x:c r="D1" s="82" t="str">
         <x:v>Telefono *</x:v>
       </x:c>
-      <x:c r="E1" s="73" t="str">
+      <x:c r="E1" s="65" t="str">
         <x:v>Ruolo</x:v>
       </x:c>
-      <x:c r="F1" s="73" t="str">
+      <x:c r="F1" s="65" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="G1" s="73" t="str">
+      <x:c r="G1" s="65" t="str">
         <x:v>Documento iniziale</x:v>
       </x:c>
-      <x:c r="H1" s="73" t="str">
+      <x:c r="H1" s="65" t="str">
         <x:v>Scadenza documento</x:v>
       </x:c>
-      <x:c r="I1" s="73" t="str">
+      <x:c r="I1" s="65" t="str">
         <x:v>Numero documento</x:v>
       </x:c>
-      <x:c r="J1" s="73" t="str">
+      <x:c r="J1" s="65" t="str">
         <x:v>Visibile in app</x:v>
       </x:c>
-      <x:c r="K1" s="74" t="str">
+      <x:c r="K1" s="66" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="75" t="str">
+      <x:c r="A2" s="67" t="str">
         <x:v>Mario Rossi</x:v>
       </x:c>
-      <x:c r="B2" s="76" t="str">
+      <x:c r="B2" s="83" t="str">
         <x:v>mario.rossi</x:v>
       </x:c>
-      <x:c r="C2" s="76" t="str">
+      <x:c r="C2" s="83" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D2" s="76" t="str">
+      <x:c r="D2" s="83" t="str">
         <x:v>+39 333 111 1111</x:v>
       </x:c>
-      <x:c r="E2" s="77" t="str">
+      <x:c r="E2" s="68" t="str">
         <x:v>Autista bilico</x:v>
       </x:c>
-      <x:c r="F2" s="77" t="str">
+      <x:c r="F2" s="68" t="str">
         <x:v>Verona</x:v>
       </x:c>
-      <x:c r="G2" s="77" t="str">
+      <x:c r="G2" s="68" t="str">
         <x:v>Patente C+E</x:v>
       </x:c>
-      <x:c r="H2" s="77" t="str">
+      <x:c r="H2" s="68" t="str">
         <x:v>2027-05-31</x:v>
       </x:c>
-      <x:c r="I2" s="92" t="str">
+      <x:c r="I2" s="94" t="str">
         <x:v>PCE12345</x:v>
       </x:c>
-      <x:c r="J2" s="76" t="str">
+      <x:c r="J2" s="83" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="K2" s="78" t="str">
+      <x:c r="K2" s="69" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="79" t="str">
+      <x:c r="A3" s="70" t="str">
         <x:v>Anna Verdi</x:v>
       </x:c>
-      <x:c r="B3" s="80" t="str">
+      <x:c r="B3" s="84" t="str">
         <x:v>anna.verdi</x:v>
       </x:c>
-      <x:c r="C3" s="80" t="str">
+      <x:c r="C3" s="84" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D3" s="80" t="str">
+      <x:c r="D3" s="84" t="str">
         <x:v>+39 333 222 2222</x:v>
       </x:c>
-      <x:c r="E3" s="81" t="str">
+      <x:c r="E3" s="71" t="str">
         <x:v>Autista furgone</x:v>
       </x:c>
-      <x:c r="F3" s="81" t="str">
+      <x:c r="F3" s="71" t="str">
         <x:v>Milano</x:v>
       </x:c>
-      <x:c r="G3" s="81" t="str">
+      <x:c r="G3" s="71" t="str">
         <x:v>CQC</x:v>
       </x:c>
-      <x:c r="H3" s="81" t="str">
+      <x:c r="H3" s="71" t="str">
         <x:v>2027-11-30</x:v>
       </x:c>
-      <x:c r="I3" s="93" t="str">
+      <x:c r="I3" s="95" t="str">
         <x:v>CQC9988</x:v>
       </x:c>
-      <x:c r="J3" s="80" t="str">
+      <x:c r="J3" s="84" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="K3" s="82" t="str"/>
+      <x:c r="K3" s="72" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="B4" s="45"/>
-      <x:c r="C4" s="45"/>
-      <x:c r="D4" s="45"/>
-      <x:c r="I4" s="94"/>
-      <x:c r="J4" s="45"/>
+      <x:c r="B4" s="73"/>
+      <x:c r="C4" s="73"/>
+      <x:c r="D4" s="73"/>
+      <x:c r="I4" s="96"/>
+      <x:c r="J4" s="73"/>
     </x:row>
     <x:row r="5">
-      <x:c r="B5" s="45"/>
-      <x:c r="C5" s="45"/>
-      <x:c r="D5" s="45"/>
-      <x:c r="I5" s="94"/>
-      <x:c r="J5" s="45"/>
+      <x:c r="B5" s="73"/>
+      <x:c r="C5" s="73"/>
+      <x:c r="D5" s="73"/>
+      <x:c r="I5" s="96"/>
+      <x:c r="J5" s="73"/>
     </x:row>
     <x:row r="6">
-      <x:c r="B6" s="45"/>
-      <x:c r="C6" s="45"/>
-      <x:c r="D6" s="45"/>
-      <x:c r="I6" s="94"/>
-      <x:c r="J6" s="45"/>
+      <x:c r="B6" s="73"/>
+      <x:c r="C6" s="73"/>
+      <x:c r="D6" s="73"/>
+      <x:c r="I6" s="96"/>
+      <x:c r="J6" s="73"/>
     </x:row>
     <x:row r="7">
-      <x:c r="B7" s="45"/>
-      <x:c r="C7" s="45"/>
-      <x:c r="D7" s="45"/>
-      <x:c r="I7" s="94"/>
-      <x:c r="J7" s="45"/>
+      <x:c r="B7" s="73"/>
+      <x:c r="C7" s="73"/>
+      <x:c r="D7" s="73"/>
+      <x:c r="I7" s="96"/>
+      <x:c r="J7" s="73"/>
     </x:row>
     <x:row r="8">
-      <x:c r="B8" s="45"/>
-      <x:c r="C8" s="45"/>
-      <x:c r="D8" s="45"/>
-      <x:c r="I8" s="94"/>
-      <x:c r="J8" s="45"/>
+      <x:c r="B8" s="73"/>
+      <x:c r="C8" s="73"/>
+      <x:c r="D8" s="73"/>
+      <x:c r="I8" s="96"/>
+      <x:c r="J8" s="73"/>
     </x:row>
     <x:row r="9">
-      <x:c r="B9" s="45"/>
-      <x:c r="C9" s="45"/>
-      <x:c r="D9" s="45"/>
-      <x:c r="I9" s="94"/>
-      <x:c r="J9" s="45"/>
+      <x:c r="B9" s="73"/>
+      <x:c r="C9" s="73"/>
+      <x:c r="D9" s="73"/>
+      <x:c r="I9" s="96"/>
+      <x:c r="J9" s="73"/>
     </x:row>
     <x:row r="10">
-      <x:c r="B10" s="45"/>
-      <x:c r="C10" s="45"/>
-      <x:c r="D10" s="45"/>
-      <x:c r="I10" s="94"/>
-      <x:c r="J10" s="45"/>
+      <x:c r="B10" s="73"/>
+      <x:c r="C10" s="73"/>
+      <x:c r="D10" s="73"/>
+      <x:c r="I10" s="96"/>
+      <x:c r="J10" s="73"/>
     </x:row>
     <x:row r="11">
-      <x:c r="B11" s="45"/>
-      <x:c r="C11" s="45"/>
-      <x:c r="D11" s="45"/>
-      <x:c r="I11" s="94"/>
-      <x:c r="J11" s="45"/>
+      <x:c r="B11" s="73"/>
+      <x:c r="C11" s="73"/>
+      <x:c r="D11" s="73"/>
+      <x:c r="I11" s="96"/>
+      <x:c r="J11" s="73"/>
     </x:row>
     <x:row r="12">
-      <x:c r="B12" s="45"/>
-      <x:c r="C12" s="45"/>
-      <x:c r="D12" s="45"/>
-      <x:c r="I12" s="94"/>
-      <x:c r="J12" s="45"/>
+      <x:c r="B12" s="73"/>
+      <x:c r="C12" s="73"/>
+      <x:c r="D12" s="73"/>
+      <x:c r="I12" s="96"/>
+      <x:c r="J12" s="73"/>
     </x:row>
     <x:row r="13">
-      <x:c r="B13" s="45"/>
-      <x:c r="C13" s="45"/>
-      <x:c r="D13" s="45"/>
-      <x:c r="I13" s="94"/>
-      <x:c r="J13" s="45"/>
+      <x:c r="B13" s="73"/>
+      <x:c r="C13" s="73"/>
+      <x:c r="D13" s="73"/>
+      <x:c r="I13" s="96"/>
+      <x:c r="J13" s="73"/>
     </x:row>
     <x:row r="14">
-      <x:c r="B14" s="45"/>
-      <x:c r="C14" s="45"/>
-      <x:c r="D14" s="45"/>
-      <x:c r="I14" s="94"/>
-      <x:c r="J14" s="45"/>
+      <x:c r="B14" s="73"/>
+      <x:c r="C14" s="73"/>
+      <x:c r="D14" s="73"/>
+      <x:c r="I14" s="96"/>
+      <x:c r="J14" s="73"/>
     </x:row>
     <x:row r="15">
-      <x:c r="B15" s="45"/>
-      <x:c r="C15" s="45"/>
-      <x:c r="D15" s="45"/>
-      <x:c r="I15" s="94"/>
-      <x:c r="J15" s="45"/>
+      <x:c r="B15" s="73"/>
+      <x:c r="C15" s="73"/>
+      <x:c r="D15" s="73"/>
+      <x:c r="I15" s="96"/>
+      <x:c r="J15" s="73"/>
     </x:row>
     <x:row r="16">
-      <x:c r="B16" s="45"/>
-      <x:c r="C16" s="45"/>
-      <x:c r="D16" s="45"/>
-      <x:c r="I16" s="94"/>
-      <x:c r="J16" s="45"/>
+      <x:c r="B16" s="73"/>
+      <x:c r="C16" s="73"/>
+      <x:c r="D16" s="73"/>
+      <x:c r="I16" s="96"/>
+      <x:c r="J16" s="73"/>
     </x:row>
     <x:row r="17">
-      <x:c r="B17" s="45"/>
-      <x:c r="C17" s="45"/>
-      <x:c r="D17" s="45"/>
-      <x:c r="I17" s="94"/>
-      <x:c r="J17" s="45"/>
+      <x:c r="B17" s="73"/>
+      <x:c r="C17" s="73"/>
+      <x:c r="D17" s="73"/>
+      <x:c r="I17" s="96"/>
+      <x:c r="J17" s="73"/>
     </x:row>
     <x:row r="18">
-      <x:c r="B18" s="45"/>
-      <x:c r="C18" s="45"/>
-      <x:c r="D18" s="45"/>
-      <x:c r="I18" s="94"/>
-      <x:c r="J18" s="45"/>
+      <x:c r="B18" s="73"/>
+      <x:c r="C18" s="73"/>
+      <x:c r="D18" s="73"/>
+      <x:c r="I18" s="96"/>
+      <x:c r="J18" s="73"/>
     </x:row>
     <x:row r="19">
-      <x:c r="B19" s="45"/>
-      <x:c r="C19" s="45"/>
-      <x:c r="D19" s="45"/>
-      <x:c r="I19" s="94"/>
-      <x:c r="J19" s="45"/>
+      <x:c r="B19" s="73"/>
+      <x:c r="C19" s="73"/>
+      <x:c r="D19" s="73"/>
+      <x:c r="I19" s="96"/>
+      <x:c r="J19" s="73"/>
     </x:row>
     <x:row r="20">
-      <x:c r="B20" s="45"/>
-      <x:c r="C20" s="45"/>
-      <x:c r="D20" s="45"/>
-      <x:c r="I20" s="94"/>
-      <x:c r="J20" s="45"/>
+      <x:c r="B20" s="73"/>
+      <x:c r="C20" s="73"/>
+      <x:c r="D20" s="73"/>
+      <x:c r="I20" s="96"/>
+      <x:c r="J20" s="73"/>
     </x:row>
     <x:row r="21">
-      <x:c r="B21" s="45"/>
-      <x:c r="C21" s="45"/>
-      <x:c r="D21" s="45"/>
-      <x:c r="I21" s="94"/>
-      <x:c r="J21" s="45"/>
+      <x:c r="B21" s="73"/>
+      <x:c r="C21" s="73"/>
+      <x:c r="D21" s="73"/>
+      <x:c r="I21" s="96"/>
+      <x:c r="J21" s="73"/>
     </x:row>
     <x:row r="22">
-      <x:c r="B22" s="45"/>
-      <x:c r="C22" s="45"/>
-      <x:c r="D22" s="45"/>
-      <x:c r="I22" s="94"/>
-      <x:c r="J22" s="45"/>
+      <x:c r="B22" s="73"/>
+      <x:c r="C22" s="73"/>
+      <x:c r="D22" s="73"/>
+      <x:c r="I22" s="96"/>
+      <x:c r="J22" s="73"/>
     </x:row>
     <x:row r="23">
-      <x:c r="B23" s="45"/>
-      <x:c r="C23" s="45"/>
-      <x:c r="D23" s="45"/>
-      <x:c r="I23" s="94"/>
-      <x:c r="J23" s="45"/>
+      <x:c r="B23" s="73"/>
+      <x:c r="C23" s="73"/>
+      <x:c r="D23" s="73"/>
+      <x:c r="I23" s="96"/>
+      <x:c r="J23" s="73"/>
     </x:row>
     <x:row r="24">
-      <x:c r="B24" s="45"/>
-      <x:c r="C24" s="45"/>
-      <x:c r="D24" s="45"/>
-      <x:c r="I24" s="94"/>
-      <x:c r="J24" s="45"/>
+      <x:c r="B24" s="73"/>
+      <x:c r="C24" s="73"/>
+      <x:c r="D24" s="73"/>
+      <x:c r="I24" s="96"/>
+      <x:c r="J24" s="73"/>
     </x:row>
     <x:row r="25">
-      <x:c r="B25" s="45"/>
-      <x:c r="C25" s="45"/>
-      <x:c r="D25" s="45"/>
-      <x:c r="I25" s="94"/>
-      <x:c r="J25" s="45"/>
+      <x:c r="B25" s="73"/>
+      <x:c r="C25" s="73"/>
+      <x:c r="D25" s="73"/>
+      <x:c r="I25" s="96"/>
+      <x:c r="J25" s="73"/>
     </x:row>
     <x:row r="26">
-      <x:c r="B26" s="45"/>
-      <x:c r="C26" s="45"/>
-      <x:c r="D26" s="45"/>
-      <x:c r="I26" s="94"/>
-      <x:c r="J26" s="45"/>
+      <x:c r="B26" s="73"/>
+      <x:c r="C26" s="73"/>
+      <x:c r="D26" s="73"/>
+      <x:c r="I26" s="96"/>
+      <x:c r="J26" s="73"/>
     </x:row>
     <x:row r="27">
-      <x:c r="B27" s="45"/>
-      <x:c r="C27" s="45"/>
-      <x:c r="D27" s="45"/>
-      <x:c r="I27" s="94"/>
-      <x:c r="J27" s="45"/>
+      <x:c r="B27" s="73"/>
+      <x:c r="C27" s="73"/>
+      <x:c r="D27" s="73"/>
+      <x:c r="I27" s="96"/>
+      <x:c r="J27" s="73"/>
     </x:row>
     <x:row r="28">
-      <x:c r="B28" s="45"/>
-      <x:c r="C28" s="45"/>
-      <x:c r="D28" s="45"/>
-      <x:c r="I28" s="94"/>
-      <x:c r="J28" s="45"/>
+      <x:c r="B28" s="73"/>
+      <x:c r="C28" s="73"/>
+      <x:c r="D28" s="73"/>
+      <x:c r="I28" s="96"/>
+      <x:c r="J28" s="73"/>
     </x:row>
     <x:row r="29">
-      <x:c r="B29" s="45"/>
-      <x:c r="C29" s="45"/>
-      <x:c r="D29" s="45"/>
-      <x:c r="I29" s="94"/>
-      <x:c r="J29" s="45"/>
+      <x:c r="B29" s="73"/>
+      <x:c r="C29" s="73"/>
+      <x:c r="D29" s="73"/>
+      <x:c r="I29" s="96"/>
+      <x:c r="J29" s="73"/>
     </x:row>
     <x:row r="30">
-      <x:c r="B30" s="45"/>
-      <x:c r="C30" s="45"/>
-      <x:c r="D30" s="45"/>
-      <x:c r="I30" s="94"/>
-      <x:c r="J30" s="45"/>
+      <x:c r="B30" s="73"/>
+      <x:c r="C30" s="73"/>
+      <x:c r="D30" s="73"/>
+      <x:c r="I30" s="96"/>
+      <x:c r="J30" s="73"/>
     </x:row>
     <x:row r="31">
-      <x:c r="B31" s="45"/>
-      <x:c r="C31" s="45"/>
-      <x:c r="D31" s="45"/>
-      <x:c r="I31" s="94"/>
-      <x:c r="J31" s="45"/>
+      <x:c r="B31" s="73"/>
+      <x:c r="C31" s="73"/>
+      <x:c r="D31" s="73"/>
+      <x:c r="I31" s="96"/>
+      <x:c r="J31" s="73"/>
     </x:row>
     <x:row r="32">
-      <x:c r="B32" s="45"/>
-      <x:c r="C32" s="45"/>
-      <x:c r="D32" s="45"/>
-      <x:c r="I32" s="94"/>
-      <x:c r="J32" s="45"/>
+      <x:c r="B32" s="73"/>
+      <x:c r="C32" s="73"/>
+      <x:c r="D32" s="73"/>
+      <x:c r="I32" s="96"/>
+      <x:c r="J32" s="73"/>
     </x:row>
     <x:row r="33">
-      <x:c r="B33" s="45"/>
-      <x:c r="C33" s="45"/>
-      <x:c r="D33" s="45"/>
-      <x:c r="I33" s="94"/>
-      <x:c r="J33" s="45"/>
+      <x:c r="B33" s="73"/>
+      <x:c r="C33" s="73"/>
+      <x:c r="D33" s="73"/>
+      <x:c r="I33" s="96"/>
+      <x:c r="J33" s="73"/>
     </x:row>
     <x:row r="34">
-      <x:c r="B34" s="45"/>
-      <x:c r="C34" s="45"/>
-      <x:c r="D34" s="45"/>
-      <x:c r="I34" s="94"/>
-      <x:c r="J34" s="45"/>
+      <x:c r="B34" s="73"/>
+      <x:c r="C34" s="73"/>
+      <x:c r="D34" s="73"/>
+      <x:c r="I34" s="96"/>
+      <x:c r="J34" s="73"/>
     </x:row>
     <x:row r="35">
-      <x:c r="B35" s="45"/>
-      <x:c r="C35" s="45"/>
-      <x:c r="D35" s="45"/>
-      <x:c r="I35" s="94"/>
-      <x:c r="J35" s="45"/>
+      <x:c r="B35" s="73"/>
+      <x:c r="C35" s="73"/>
+      <x:c r="D35" s="73"/>
+      <x:c r="I35" s="96"/>
+      <x:c r="J35" s="73"/>
     </x:row>
     <x:row r="36">
-      <x:c r="B36" s="45"/>
-      <x:c r="C36" s="45"/>
-      <x:c r="D36" s="45"/>
-      <x:c r="I36" s="94"/>
-      <x:c r="J36" s="45"/>
+      <x:c r="B36" s="73"/>
+      <x:c r="C36" s="73"/>
+      <x:c r="D36" s="73"/>
+      <x:c r="I36" s="96"/>
+      <x:c r="J36" s="73"/>
     </x:row>
     <x:row r="37">
-      <x:c r="B37" s="45"/>
-      <x:c r="C37" s="45"/>
-      <x:c r="D37" s="45"/>
-      <x:c r="I37" s="94"/>
-      <x:c r="J37" s="45"/>
+      <x:c r="B37" s="73"/>
+      <x:c r="C37" s="73"/>
+      <x:c r="D37" s="73"/>
+      <x:c r="I37" s="96"/>
+      <x:c r="J37" s="73"/>
     </x:row>
     <x:row r="38">
-      <x:c r="B38" s="45"/>
-      <x:c r="C38" s="45"/>
-      <x:c r="D38" s="45"/>
-      <x:c r="I38" s="94"/>
-      <x:c r="J38" s="45"/>
+      <x:c r="B38" s="73"/>
+      <x:c r="C38" s="73"/>
+      <x:c r="D38" s="73"/>
+      <x:c r="I38" s="96"/>
+      <x:c r="J38" s="73"/>
     </x:row>
     <x:row r="39">
-      <x:c r="B39" s="45"/>
-      <x:c r="C39" s="45"/>
-      <x:c r="D39" s="45"/>
-      <x:c r="I39" s="94"/>
-      <x:c r="J39" s="45"/>
+      <x:c r="B39" s="73"/>
+      <x:c r="C39" s="73"/>
+      <x:c r="D39" s="73"/>
+      <x:c r="I39" s="96"/>
+      <x:c r="J39" s="73"/>
     </x:row>
     <x:row r="40">
-      <x:c r="B40" s="45"/>
-      <x:c r="C40" s="45"/>
-      <x:c r="D40" s="45"/>
-      <x:c r="I40" s="94"/>
-      <x:c r="J40" s="45"/>
+      <x:c r="B40" s="73"/>
+      <x:c r="C40" s="73"/>
+      <x:c r="D40" s="73"/>
+      <x:c r="I40" s="96"/>
+      <x:c r="J40" s="73"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1261,12 +2175,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83ecd371c6a14f08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R053b1b7a7b5a4dba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1283,283 +2197,283 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="71" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Nome e cognome *</x:v>
       </x:c>
-      <x:c r="B1" s="72" t="str">
+      <x:c r="B1" s="82" t="str">
         <x:v>Username *</x:v>
       </x:c>
-      <x:c r="C1" s="72" t="str">
+      <x:c r="C1" s="82" t="str">
         <x:v>Password *</x:v>
       </x:c>
-      <x:c r="D1" s="73" t="str">
+      <x:c r="D1" s="65" t="str">
         <x:v>Telefono</x:v>
       </x:c>
-      <x:c r="E1" s="73" t="str">
+      <x:c r="E1" s="65" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="F1" s="73" t="str">
+      <x:c r="F1" s="65" t="str">
         <x:v>Reparto</x:v>
       </x:c>
-      <x:c r="G1" s="73" t="str">
+      <x:c r="G1" s="65" t="str">
         <x:v>Ruolo</x:v>
       </x:c>
-      <x:c r="H1" s="73" t="str">
+      <x:c r="H1" s="65" t="str">
         <x:v>Mansione</x:v>
       </x:c>
-      <x:c r="I1" s="73" t="str">
+      <x:c r="I1" s="65" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="J1" s="74" t="str">
+      <x:c r="J1" s="66" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="75" t="str">
+      <x:c r="A2" s="67" t="str">
         <x:v>Paola Bianchi</x:v>
       </x:c>
-      <x:c r="B2" s="76" t="str">
+      <x:c r="B2" s="83" t="str">
         <x:v>paola.bianchi</x:v>
       </x:c>
-      <x:c r="C2" s="76" t="str">
+      <x:c r="C2" s="83" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D2" s="76" t="str">
+      <x:c r="D2" s="83" t="str">
         <x:v>+39 333 444 4444</x:v>
       </x:c>
-      <x:c r="E2" s="77" t="str">
+      <x:c r="E2" s="68" t="str">
         <x:v>paola.bianchi@azienda.it</x:v>
       </x:c>
-      <x:c r="F2" s="77" t="str">
+      <x:c r="F2" s="68" t="str">
         <x:v>ufficio</x:v>
       </x:c>
-      <x:c r="G2" s="77" t="str">
+      <x:c r="G2" s="68" t="str">
         <x:v>Impiegato ufficio</x:v>
       </x:c>
-      <x:c r="H2" s="77" t="str">
+      <x:c r="H2" s="68" t="str">
         <x:v>Ufficio traffico</x:v>
       </x:c>
-      <x:c r="I2" s="77" t="str">
+      <x:c r="I2" s="68" t="str">
         <x:v>Sede centrale</x:v>
       </x:c>
-      <x:c r="J2" s="78" t="str">
+      <x:c r="J2" s="69" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="79" t="str">
+      <x:c r="A3" s="70" t="str">
         <x:v>Luca Neri</x:v>
       </x:c>
-      <x:c r="B3" s="80" t="str">
+      <x:c r="B3" s="84" t="str">
         <x:v>luca.neri</x:v>
       </x:c>
-      <x:c r="C3" s="80" t="str">
+      <x:c r="C3" s="84" t="str">
         <x:v>Vygo2026!</x:v>
       </x:c>
-      <x:c r="D3" s="80" t="str">
+      <x:c r="D3" s="84" t="str">
         <x:v>+39 333 555 5555</x:v>
       </x:c>
-      <x:c r="E3" s="81" t="str">
+      <x:c r="E3" s="71" t="str">
         <x:v>luca.neri@azienda.it</x:v>
       </x:c>
-      <x:c r="F3" s="81" t="str">
+      <x:c r="F3" s="71" t="str">
         <x:v>magazzino</x:v>
       </x:c>
-      <x:c r="G3" s="81" t="str">
+      <x:c r="G3" s="71" t="str">
         <x:v>Carrellista</x:v>
       </x:c>
-      <x:c r="H3" s="81" t="str">
+      <x:c r="H3" s="71" t="str">
         <x:v>Capo turno magazzino</x:v>
       </x:c>
-      <x:c r="I3" s="81" t="str">
+      <x:c r="I3" s="71" t="str">
         <x:v>Magazzino A</x:v>
       </x:c>
-      <x:c r="J3" s="82" t="str"/>
+      <x:c r="J3" s="72" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="B4" s="45"/>
-      <x:c r="C4" s="45"/>
-      <x:c r="D4" s="45"/>
+      <x:c r="B4" s="73"/>
+      <x:c r="C4" s="73"/>
+      <x:c r="D4" s="73"/>
     </x:row>
     <x:row r="5">
-      <x:c r="B5" s="45"/>
-      <x:c r="C5" s="45"/>
-      <x:c r="D5" s="45"/>
+      <x:c r="B5" s="73"/>
+      <x:c r="C5" s="73"/>
+      <x:c r="D5" s="73"/>
     </x:row>
     <x:row r="6">
-      <x:c r="B6" s="45"/>
-      <x:c r="C6" s="45"/>
-      <x:c r="D6" s="45"/>
+      <x:c r="B6" s="73"/>
+      <x:c r="C6" s="73"/>
+      <x:c r="D6" s="73"/>
     </x:row>
     <x:row r="7">
-      <x:c r="B7" s="45"/>
-      <x:c r="C7" s="45"/>
-      <x:c r="D7" s="45"/>
+      <x:c r="B7" s="73"/>
+      <x:c r="C7" s="73"/>
+      <x:c r="D7" s="73"/>
     </x:row>
     <x:row r="8">
-      <x:c r="B8" s="45"/>
-      <x:c r="C8" s="45"/>
-      <x:c r="D8" s="45"/>
+      <x:c r="B8" s="73"/>
+      <x:c r="C8" s="73"/>
+      <x:c r="D8" s="73"/>
     </x:row>
     <x:row r="9">
-      <x:c r="B9" s="45"/>
-      <x:c r="C9" s="45"/>
-      <x:c r="D9" s="45"/>
+      <x:c r="B9" s="73"/>
+      <x:c r="C9" s="73"/>
+      <x:c r="D9" s="73"/>
     </x:row>
     <x:row r="10">
-      <x:c r="B10" s="45"/>
-      <x:c r="C10" s="45"/>
-      <x:c r="D10" s="45"/>
+      <x:c r="B10" s="73"/>
+      <x:c r="C10" s="73"/>
+      <x:c r="D10" s="73"/>
     </x:row>
     <x:row r="11">
-      <x:c r="B11" s="45"/>
-      <x:c r="C11" s="45"/>
-      <x:c r="D11" s="45"/>
+      <x:c r="B11" s="73"/>
+      <x:c r="C11" s="73"/>
+      <x:c r="D11" s="73"/>
     </x:row>
     <x:row r="12">
-      <x:c r="B12" s="45"/>
-      <x:c r="C12" s="45"/>
-      <x:c r="D12" s="45"/>
+      <x:c r="B12" s="73"/>
+      <x:c r="C12" s="73"/>
+      <x:c r="D12" s="73"/>
     </x:row>
     <x:row r="13">
-      <x:c r="B13" s="45"/>
-      <x:c r="C13" s="45"/>
-      <x:c r="D13" s="45"/>
+      <x:c r="B13" s="73"/>
+      <x:c r="C13" s="73"/>
+      <x:c r="D13" s="73"/>
     </x:row>
     <x:row r="14">
-      <x:c r="B14" s="45"/>
-      <x:c r="C14" s="45"/>
-      <x:c r="D14" s="45"/>
+      <x:c r="B14" s="73"/>
+      <x:c r="C14" s="73"/>
+      <x:c r="D14" s="73"/>
     </x:row>
     <x:row r="15">
-      <x:c r="B15" s="45"/>
-      <x:c r="C15" s="45"/>
-      <x:c r="D15" s="45"/>
+      <x:c r="B15" s="73"/>
+      <x:c r="C15" s="73"/>
+      <x:c r="D15" s="73"/>
     </x:row>
     <x:row r="16">
-      <x:c r="B16" s="45"/>
-      <x:c r="C16" s="45"/>
-      <x:c r="D16" s="45"/>
+      <x:c r="B16" s="73"/>
+      <x:c r="C16" s="73"/>
+      <x:c r="D16" s="73"/>
     </x:row>
     <x:row r="17">
-      <x:c r="B17" s="45"/>
-      <x:c r="C17" s="45"/>
-      <x:c r="D17" s="45"/>
+      <x:c r="B17" s="73"/>
+      <x:c r="C17" s="73"/>
+      <x:c r="D17" s="73"/>
     </x:row>
     <x:row r="18">
-      <x:c r="B18" s="45"/>
-      <x:c r="C18" s="45"/>
-      <x:c r="D18" s="45"/>
+      <x:c r="B18" s="73"/>
+      <x:c r="C18" s="73"/>
+      <x:c r="D18" s="73"/>
     </x:row>
     <x:row r="19">
-      <x:c r="B19" s="45"/>
-      <x:c r="C19" s="45"/>
-      <x:c r="D19" s="45"/>
+      <x:c r="B19" s="73"/>
+      <x:c r="C19" s="73"/>
+      <x:c r="D19" s="73"/>
     </x:row>
     <x:row r="20">
-      <x:c r="B20" s="45"/>
-      <x:c r="C20" s="45"/>
-      <x:c r="D20" s="45"/>
+      <x:c r="B20" s="73"/>
+      <x:c r="C20" s="73"/>
+      <x:c r="D20" s="73"/>
     </x:row>
     <x:row r="21">
-      <x:c r="B21" s="45"/>
-      <x:c r="C21" s="45"/>
-      <x:c r="D21" s="45"/>
+      <x:c r="B21" s="73"/>
+      <x:c r="C21" s="73"/>
+      <x:c r="D21" s="73"/>
     </x:row>
     <x:row r="22">
-      <x:c r="B22" s="45"/>
-      <x:c r="C22" s="45"/>
-      <x:c r="D22" s="45"/>
+      <x:c r="B22" s="73"/>
+      <x:c r="C22" s="73"/>
+      <x:c r="D22" s="73"/>
     </x:row>
     <x:row r="23">
-      <x:c r="B23" s="45"/>
-      <x:c r="C23" s="45"/>
-      <x:c r="D23" s="45"/>
+      <x:c r="B23" s="73"/>
+      <x:c r="C23" s="73"/>
+      <x:c r="D23" s="73"/>
     </x:row>
     <x:row r="24">
-      <x:c r="B24" s="45"/>
-      <x:c r="C24" s="45"/>
-      <x:c r="D24" s="45"/>
+      <x:c r="B24" s="73"/>
+      <x:c r="C24" s="73"/>
+      <x:c r="D24" s="73"/>
     </x:row>
     <x:row r="25">
-      <x:c r="B25" s="45"/>
-      <x:c r="C25" s="45"/>
-      <x:c r="D25" s="45"/>
+      <x:c r="B25" s="73"/>
+      <x:c r="C25" s="73"/>
+      <x:c r="D25" s="73"/>
     </x:row>
     <x:row r="26">
-      <x:c r="B26" s="45"/>
-      <x:c r="C26" s="45"/>
-      <x:c r="D26" s="45"/>
+      <x:c r="B26" s="73"/>
+      <x:c r="C26" s="73"/>
+      <x:c r="D26" s="73"/>
     </x:row>
     <x:row r="27">
-      <x:c r="B27" s="45"/>
-      <x:c r="C27" s="45"/>
-      <x:c r="D27" s="45"/>
+      <x:c r="B27" s="73"/>
+      <x:c r="C27" s="73"/>
+      <x:c r="D27" s="73"/>
     </x:row>
     <x:row r="28">
-      <x:c r="B28" s="45"/>
-      <x:c r="C28" s="45"/>
-      <x:c r="D28" s="45"/>
+      <x:c r="B28" s="73"/>
+      <x:c r="C28" s="73"/>
+      <x:c r="D28" s="73"/>
     </x:row>
     <x:row r="29">
-      <x:c r="B29" s="45"/>
-      <x:c r="C29" s="45"/>
-      <x:c r="D29" s="45"/>
+      <x:c r="B29" s="73"/>
+      <x:c r="C29" s="73"/>
+      <x:c r="D29" s="73"/>
     </x:row>
     <x:row r="30">
-      <x:c r="B30" s="45"/>
-      <x:c r="C30" s="45"/>
-      <x:c r="D30" s="45"/>
+      <x:c r="B30" s="73"/>
+      <x:c r="C30" s="73"/>
+      <x:c r="D30" s="73"/>
     </x:row>
     <x:row r="31">
-      <x:c r="B31" s="45"/>
-      <x:c r="C31" s="45"/>
-      <x:c r="D31" s="45"/>
+      <x:c r="B31" s="73"/>
+      <x:c r="C31" s="73"/>
+      <x:c r="D31" s="73"/>
     </x:row>
     <x:row r="32">
-      <x:c r="B32" s="45"/>
-      <x:c r="C32" s="45"/>
-      <x:c r="D32" s="45"/>
+      <x:c r="B32" s="73"/>
+      <x:c r="C32" s="73"/>
+      <x:c r="D32" s="73"/>
     </x:row>
     <x:row r="33">
-      <x:c r="B33" s="45"/>
-      <x:c r="C33" s="45"/>
-      <x:c r="D33" s="45"/>
+      <x:c r="B33" s="73"/>
+      <x:c r="C33" s="73"/>
+      <x:c r="D33" s="73"/>
     </x:row>
     <x:row r="34">
-      <x:c r="B34" s="45"/>
-      <x:c r="C34" s="45"/>
-      <x:c r="D34" s="45"/>
+      <x:c r="B34" s="73"/>
+      <x:c r="C34" s="73"/>
+      <x:c r="D34" s="73"/>
     </x:row>
     <x:row r="35">
-      <x:c r="B35" s="45"/>
-      <x:c r="C35" s="45"/>
-      <x:c r="D35" s="45"/>
+      <x:c r="B35" s="73"/>
+      <x:c r="C35" s="73"/>
+      <x:c r="D35" s="73"/>
     </x:row>
     <x:row r="36">
-      <x:c r="B36" s="45"/>
-      <x:c r="C36" s="45"/>
-      <x:c r="D36" s="45"/>
+      <x:c r="B36" s="73"/>
+      <x:c r="C36" s="73"/>
+      <x:c r="D36" s="73"/>
     </x:row>
     <x:row r="37">
-      <x:c r="B37" s="45"/>
-      <x:c r="C37" s="45"/>
-      <x:c r="D37" s="45"/>
+      <x:c r="B37" s="73"/>
+      <x:c r="C37" s="73"/>
+      <x:c r="D37" s="73"/>
     </x:row>
     <x:row r="38">
-      <x:c r="B38" s="45"/>
-      <x:c r="C38" s="45"/>
-      <x:c r="D38" s="45"/>
+      <x:c r="B38" s="73"/>
+      <x:c r="C38" s="73"/>
+      <x:c r="D38" s="73"/>
     </x:row>
     <x:row r="39">
-      <x:c r="B39" s="45"/>
-      <x:c r="C39" s="45"/>
-      <x:c r="D39" s="45"/>
+      <x:c r="B39" s="73"/>
+      <x:c r="C39" s="73"/>
+      <x:c r="D39" s="73"/>
     </x:row>
     <x:row r="40">
-      <x:c r="B40" s="45"/>
-      <x:c r="C40" s="45"/>
-      <x:c r="D40" s="45"/>
+      <x:c r="B40" s="73"/>
+      <x:c r="C40" s="73"/>
+      <x:c r="D40" s="73"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -1572,12 +2486,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfe4ae7da9064f99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1686d31872d4e47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1591,236 +2505,236 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="71" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Targa *</x:v>
       </x:c>
-      <x:c r="B1" s="73" t="str">
+      <x:c r="B1" s="65" t="str">
         <x:v>Categoria mezzo</x:v>
       </x:c>
-      <x:c r="C1" s="73" t="str">
+      <x:c r="C1" s="65" t="str">
         <x:v>Modello</x:v>
       </x:c>
-      <x:c r="D1" s="73" t="str">
+      <x:c r="D1" s="65" t="str">
         <x:v>Allestimento</x:v>
       </x:c>
-      <x:c r="E1" s="73" t="str">
+      <x:c r="E1" s="65" t="str">
         <x:v>KM</x:v>
       </x:c>
-      <x:c r="F1" s="73" t="str">
+      <x:c r="F1" s="65" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="G1" s="74" t="str">
+      <x:c r="G1" s="66" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="87" t="str">
+      <x:c r="A2" s="89" t="str">
         <x:v>AB123CD</x:v>
       </x:c>
-      <x:c r="B2" s="77" t="str">
+      <x:c r="B2" s="68" t="str">
         <x:v>trattore</x:v>
       </x:c>
-      <x:c r="C2" s="77" t="str">
+      <x:c r="C2" s="68" t="str">
         <x:v>Volvo FH</x:v>
       </x:c>
-      <x:c r="D2" s="77" t="str">
+      <x:c r="D2" s="68" t="str">
         <x:v>Trattore stradale</x:v>
       </x:c>
-      <x:c r="E2" s="89" t="n">
+      <x:c r="E2" s="91" t="n">
         <x:v>340000</x:v>
       </x:c>
-      <x:c r="F2" s="77" t="str">
+      <x:c r="F2" s="68" t="str">
         <x:v>Verona</x:v>
       </x:c>
-      <x:c r="G2" s="78" t="str">
+      <x:c r="G2" s="69" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="87" t="str">
+      <x:c r="A3" s="89" t="str">
         <x:v>SR456EF</x:v>
       </x:c>
-      <x:c r="B3" s="77" t="str">
+      <x:c r="B3" s="68" t="str">
         <x:v>semirimorchio</x:v>
       </x:c>
-      <x:c r="C3" s="77" t="str">
+      <x:c r="C3" s="68" t="str">
         <x:v>Krone</x:v>
       </x:c>
-      <x:c r="D3" s="77" t="str">
+      <x:c r="D3" s="68" t="str">
         <x:v>Centinato</x:v>
       </x:c>
-      <x:c r="E3" s="89" t="n">
+      <x:c r="E3" s="91" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F3" s="77" t="str">
+      <x:c r="F3" s="68" t="str">
         <x:v>Verona</x:v>
       </x:c>
-      <x:c r="G3" s="78" t="str"/>
+      <x:c r="G3" s="69" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="88" t="str">
+      <x:c r="A4" s="90" t="str">
         <x:v>FG789HI</x:v>
       </x:c>
-      <x:c r="B4" s="81" t="str">
+      <x:c r="B4" s="71" t="str">
         <x:v>furgone</x:v>
       </x:c>
-      <x:c r="C4" s="81" t="str">
+      <x:c r="C4" s="71" t="str">
         <x:v>Iveco Daily</x:v>
       </x:c>
-      <x:c r="D4" s="81" t="str">
+      <x:c r="D4" s="71" t="str">
         <x:v>Furgone cassonato</x:v>
       </x:c>
-      <x:c r="E4" s="90" t="n">
+      <x:c r="E4" s="92" t="n">
         <x:v>82000</x:v>
       </x:c>
-      <x:c r="F4" s="81" t="str">
+      <x:c r="F4" s="71" t="str">
         <x:v>Milano</x:v>
       </x:c>
-      <x:c r="G4" s="82" t="str"/>
+      <x:c r="G4" s="72" t="str"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="45"/>
-      <x:c r="E5" s="91"/>
+      <x:c r="A5" s="73"/>
+      <x:c r="E5" s="93"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="45"/>
-      <x:c r="E6" s="91"/>
+      <x:c r="A6" s="73"/>
+      <x:c r="E6" s="93"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="45"/>
-      <x:c r="E7" s="91"/>
+      <x:c r="A7" s="73"/>
+      <x:c r="E7" s="93"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="45"/>
-      <x:c r="E8" s="91"/>
+      <x:c r="A8" s="73"/>
+      <x:c r="E8" s="93"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45"/>
-      <x:c r="E9" s="91"/>
+      <x:c r="A9" s="73"/>
+      <x:c r="E9" s="93"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="45"/>
-      <x:c r="E10" s="91"/>
+      <x:c r="A10" s="73"/>
+      <x:c r="E10" s="93"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="45"/>
-      <x:c r="E11" s="91"/>
+      <x:c r="A11" s="73"/>
+      <x:c r="E11" s="93"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="45"/>
-      <x:c r="E12" s="91"/>
+      <x:c r="A12" s="73"/>
+      <x:c r="E12" s="93"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="45"/>
-      <x:c r="E13" s="91"/>
+      <x:c r="A13" s="73"/>
+      <x:c r="E13" s="93"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="45"/>
-      <x:c r="E14" s="91"/>
+      <x:c r="A14" s="73"/>
+      <x:c r="E14" s="93"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="45"/>
-      <x:c r="E15" s="91"/>
+      <x:c r="A15" s="73"/>
+      <x:c r="E15" s="93"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="45"/>
-      <x:c r="E16" s="91"/>
+      <x:c r="A16" s="73"/>
+      <x:c r="E16" s="93"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="45"/>
-      <x:c r="E17" s="91"/>
+      <x:c r="A17" s="73"/>
+      <x:c r="E17" s="93"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="45"/>
-      <x:c r="E18" s="91"/>
+      <x:c r="A18" s="73"/>
+      <x:c r="E18" s="93"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="45"/>
-      <x:c r="E19" s="91"/>
+      <x:c r="A19" s="73"/>
+      <x:c r="E19" s="93"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="45"/>
-      <x:c r="E20" s="91"/>
+      <x:c r="A20" s="73"/>
+      <x:c r="E20" s="93"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="45"/>
-      <x:c r="E21" s="91"/>
+      <x:c r="A21" s="73"/>
+      <x:c r="E21" s="93"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="45"/>
-      <x:c r="E22" s="91"/>
+      <x:c r="A22" s="73"/>
+      <x:c r="E22" s="93"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="45"/>
-      <x:c r="E23" s="91"/>
+      <x:c r="A23" s="73"/>
+      <x:c r="E23" s="93"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="45"/>
-      <x:c r="E24" s="91"/>
+      <x:c r="A24" s="73"/>
+      <x:c r="E24" s="93"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="45"/>
-      <x:c r="E25" s="91"/>
+      <x:c r="A25" s="73"/>
+      <x:c r="E25" s="93"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="45"/>
-      <x:c r="E26" s="91"/>
+      <x:c r="A26" s="73"/>
+      <x:c r="E26" s="93"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="45"/>
-      <x:c r="E27" s="91"/>
+      <x:c r="A27" s="73"/>
+      <x:c r="E27" s="93"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="45"/>
-      <x:c r="E28" s="91"/>
+      <x:c r="A28" s="73"/>
+      <x:c r="E28" s="93"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="45"/>
-      <x:c r="E29" s="91"/>
+      <x:c r="A29" s="73"/>
+      <x:c r="E29" s="93"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="45"/>
-      <x:c r="E30" s="91"/>
+      <x:c r="A30" s="73"/>
+      <x:c r="E30" s="93"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="45"/>
-      <x:c r="E31" s="91"/>
+      <x:c r="A31" s="73"/>
+      <x:c r="E31" s="93"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="45"/>
-      <x:c r="E32" s="91"/>
+      <x:c r="A32" s="73"/>
+      <x:c r="E32" s="93"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="45"/>
-      <x:c r="E33" s="91"/>
+      <x:c r="A33" s="73"/>
+      <x:c r="E33" s="93"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="45"/>
-      <x:c r="E34" s="91"/>
+      <x:c r="A34" s="73"/>
+      <x:c r="E34" s="93"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="45"/>
-      <x:c r="E35" s="91"/>
+      <x:c r="A35" s="73"/>
+      <x:c r="E35" s="93"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="45"/>
-      <x:c r="E36" s="91"/>
+      <x:c r="A36" s="73"/>
+      <x:c r="E36" s="93"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="45"/>
-      <x:c r="E37" s="91"/>
+      <x:c r="A37" s="73"/>
+      <x:c r="E37" s="93"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="45"/>
-      <x:c r="E38" s="91"/>
+      <x:c r="A38" s="73"/>
+      <x:c r="E38" s="93"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="45"/>
-      <x:c r="E39" s="91"/>
+      <x:c r="A39" s="73"/>
+      <x:c r="E39" s="93"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="45"/>
-      <x:c r="E40" s="91"/>
+      <x:c r="A40" s="73"/>
+      <x:c r="E40" s="93"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -1830,12 +2744,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb48f3ac12b314391"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd161bf623688475d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1848,284 +2762,284 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="71" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Codice *</x:v>
       </x:c>
-      <x:c r="B1" s="73" t="str">
+      <x:c r="B1" s="65" t="str">
         <x:v>Tipo attrezzatura</x:v>
       </x:c>
-      <x:c r="C1" s="73" t="str">
+      <x:c r="C1" s="65" t="str">
         <x:v>Modello</x:v>
       </x:c>
-      <x:c r="D1" s="73" t="str">
+      <x:c r="D1" s="65" t="str">
         <x:v>Matricola</x:v>
       </x:c>
-      <x:c r="E1" s="73" t="str">
+      <x:c r="E1" s="65" t="str">
         <x:v>Deposito / sede</x:v>
       </x:c>
-      <x:c r="F1" s="74" t="str">
+      <x:c r="F1" s="66" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="87" t="str">
+      <x:c r="A2" s="89" t="str">
         <x:v>MUL-01</x:v>
       </x:c>
-      <x:c r="B2" s="76" t="str">
+      <x:c r="B2" s="83" t="str">
         <x:v>muletto</x:v>
       </x:c>
-      <x:c r="C2" s="76" t="str">
+      <x:c r="C2" s="83" t="str">
         <x:v>Toyota 8FB</x:v>
       </x:c>
-      <x:c r="D2" s="76" t="str">
+      <x:c r="D2" s="83" t="str">
         <x:v>MAT-987</x:v>
       </x:c>
-      <x:c r="E2" s="77" t="str">
+      <x:c r="E2" s="68" t="str">
         <x:v>Magazzino A</x:v>
       </x:c>
-      <x:c r="F2" s="78" t="str">
+      <x:c r="F2" s="69" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="88" t="str">
+      <x:c r="A3" s="90" t="str">
         <x:v>TP-02</x:v>
       </x:c>
-      <x:c r="B3" s="80" t="str">
+      <x:c r="B3" s="84" t="str">
         <x:v>transpallet</x:v>
       </x:c>
-      <x:c r="C3" s="80" t="str">
+      <x:c r="C3" s="84" t="str">
         <x:v>BT Levio</x:v>
       </x:c>
-      <x:c r="D3" s="80" t="str">
+      <x:c r="D3" s="84" t="str">
         <x:v>TP-445</x:v>
       </x:c>
-      <x:c r="E3" s="81" t="str">
+      <x:c r="E3" s="71" t="str">
         <x:v>Magazzino A</x:v>
       </x:c>
-      <x:c r="F3" s="82" t="str"/>
+      <x:c r="F3" s="72" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="45"/>
-      <x:c r="B4" s="45"/>
-      <x:c r="C4" s="45"/>
-      <x:c r="D4" s="45"/>
+      <x:c r="A4" s="73"/>
+      <x:c r="B4" s="73"/>
+      <x:c r="C4" s="73"/>
+      <x:c r="D4" s="73"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="45"/>
-      <x:c r="B5" s="45"/>
-      <x:c r="C5" s="45"/>
-      <x:c r="D5" s="45"/>
+      <x:c r="A5" s="73"/>
+      <x:c r="B5" s="73"/>
+      <x:c r="C5" s="73"/>
+      <x:c r="D5" s="73"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="45"/>
-      <x:c r="B6" s="45"/>
-      <x:c r="C6" s="45"/>
-      <x:c r="D6" s="45"/>
+      <x:c r="A6" s="73"/>
+      <x:c r="B6" s="73"/>
+      <x:c r="C6" s="73"/>
+      <x:c r="D6" s="73"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="45"/>
-      <x:c r="B7" s="45"/>
-      <x:c r="C7" s="45"/>
-      <x:c r="D7" s="45"/>
+      <x:c r="A7" s="73"/>
+      <x:c r="B7" s="73"/>
+      <x:c r="C7" s="73"/>
+      <x:c r="D7" s="73"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="45"/>
-      <x:c r="B8" s="45"/>
-      <x:c r="C8" s="45"/>
-      <x:c r="D8" s="45"/>
+      <x:c r="A8" s="73"/>
+      <x:c r="B8" s="73"/>
+      <x:c r="C8" s="73"/>
+      <x:c r="D8" s="73"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45"/>
-      <x:c r="B9" s="45"/>
-      <x:c r="C9" s="45"/>
-      <x:c r="D9" s="45"/>
+      <x:c r="A9" s="73"/>
+      <x:c r="B9" s="73"/>
+      <x:c r="C9" s="73"/>
+      <x:c r="D9" s="73"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="45"/>
-      <x:c r="B10" s="45"/>
-      <x:c r="C10" s="45"/>
-      <x:c r="D10" s="45"/>
+      <x:c r="A10" s="73"/>
+      <x:c r="B10" s="73"/>
+      <x:c r="C10" s="73"/>
+      <x:c r="D10" s="73"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="45"/>
-      <x:c r="B11" s="45"/>
-      <x:c r="C11" s="45"/>
-      <x:c r="D11" s="45"/>
+      <x:c r="A11" s="73"/>
+      <x:c r="B11" s="73"/>
+      <x:c r="C11" s="73"/>
+      <x:c r="D11" s="73"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="45"/>
-      <x:c r="B12" s="45"/>
-      <x:c r="C12" s="45"/>
-      <x:c r="D12" s="45"/>
+      <x:c r="A12" s="73"/>
+      <x:c r="B12" s="73"/>
+      <x:c r="C12" s="73"/>
+      <x:c r="D12" s="73"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="45"/>
-      <x:c r="B13" s="45"/>
-      <x:c r="C13" s="45"/>
-      <x:c r="D13" s="45"/>
+      <x:c r="A13" s="73"/>
+      <x:c r="B13" s="73"/>
+      <x:c r="C13" s="73"/>
+      <x:c r="D13" s="73"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="45"/>
-      <x:c r="B14" s="45"/>
-      <x:c r="C14" s="45"/>
-      <x:c r="D14" s="45"/>
+      <x:c r="A14" s="73"/>
+      <x:c r="B14" s="73"/>
+      <x:c r="C14" s="73"/>
+      <x:c r="D14" s="73"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="45"/>
-      <x:c r="B15" s="45"/>
-      <x:c r="C15" s="45"/>
-      <x:c r="D15" s="45"/>
+      <x:c r="A15" s="73"/>
+      <x:c r="B15" s="73"/>
+      <x:c r="C15" s="73"/>
+      <x:c r="D15" s="73"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="45"/>
-      <x:c r="B16" s="45"/>
-      <x:c r="C16" s="45"/>
-      <x:c r="D16" s="45"/>
+      <x:c r="A16" s="73"/>
+      <x:c r="B16" s="73"/>
+      <x:c r="C16" s="73"/>
+      <x:c r="D16" s="73"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="45"/>
-      <x:c r="B17" s="45"/>
-      <x:c r="C17" s="45"/>
-      <x:c r="D17" s="45"/>
+      <x:c r="A17" s="73"/>
+      <x:c r="B17" s="73"/>
+      <x:c r="C17" s="73"/>
+      <x:c r="D17" s="73"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="45"/>
-      <x:c r="B18" s="45"/>
-      <x:c r="C18" s="45"/>
-      <x:c r="D18" s="45"/>
+      <x:c r="A18" s="73"/>
+      <x:c r="B18" s="73"/>
+      <x:c r="C18" s="73"/>
+      <x:c r="D18" s="73"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="45"/>
-      <x:c r="B19" s="45"/>
-      <x:c r="C19" s="45"/>
-      <x:c r="D19" s="45"/>
+      <x:c r="A19" s="73"/>
+      <x:c r="B19" s="73"/>
+      <x:c r="C19" s="73"/>
+      <x:c r="D19" s="73"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="45"/>
-      <x:c r="B20" s="45"/>
-      <x:c r="C20" s="45"/>
-      <x:c r="D20" s="45"/>
+      <x:c r="A20" s="73"/>
+      <x:c r="B20" s="73"/>
+      <x:c r="C20" s="73"/>
+      <x:c r="D20" s="73"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="45"/>
-      <x:c r="B21" s="45"/>
-      <x:c r="C21" s="45"/>
-      <x:c r="D21" s="45"/>
+      <x:c r="A21" s="73"/>
+      <x:c r="B21" s="73"/>
+      <x:c r="C21" s="73"/>
+      <x:c r="D21" s="73"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="45"/>
-      <x:c r="B22" s="45"/>
-      <x:c r="C22" s="45"/>
-      <x:c r="D22" s="45"/>
+      <x:c r="A22" s="73"/>
+      <x:c r="B22" s="73"/>
+      <x:c r="C22" s="73"/>
+      <x:c r="D22" s="73"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="45"/>
-      <x:c r="B23" s="45"/>
-      <x:c r="C23" s="45"/>
-      <x:c r="D23" s="45"/>
+      <x:c r="A23" s="73"/>
+      <x:c r="B23" s="73"/>
+      <x:c r="C23" s="73"/>
+      <x:c r="D23" s="73"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="45"/>
-      <x:c r="B24" s="45"/>
-      <x:c r="C24" s="45"/>
-      <x:c r="D24" s="45"/>
+      <x:c r="A24" s="73"/>
+      <x:c r="B24" s="73"/>
+      <x:c r="C24" s="73"/>
+      <x:c r="D24" s="73"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="45"/>
-      <x:c r="B25" s="45"/>
-      <x:c r="C25" s="45"/>
-      <x:c r="D25" s="45"/>
+      <x:c r="A25" s="73"/>
+      <x:c r="B25" s="73"/>
+      <x:c r="C25" s="73"/>
+      <x:c r="D25" s="73"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="45"/>
-      <x:c r="B26" s="45"/>
-      <x:c r="C26" s="45"/>
-      <x:c r="D26" s="45"/>
+      <x:c r="A26" s="73"/>
+      <x:c r="B26" s="73"/>
+      <x:c r="C26" s="73"/>
+      <x:c r="D26" s="73"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="45"/>
-      <x:c r="B27" s="45"/>
-      <x:c r="C27" s="45"/>
-      <x:c r="D27" s="45"/>
+      <x:c r="A27" s="73"/>
+      <x:c r="B27" s="73"/>
+      <x:c r="C27" s="73"/>
+      <x:c r="D27" s="73"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="45"/>
-      <x:c r="B28" s="45"/>
-      <x:c r="C28" s="45"/>
-      <x:c r="D28" s="45"/>
+      <x:c r="A28" s="73"/>
+      <x:c r="B28" s="73"/>
+      <x:c r="C28" s="73"/>
+      <x:c r="D28" s="73"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="45"/>
-      <x:c r="B29" s="45"/>
-      <x:c r="C29" s="45"/>
-      <x:c r="D29" s="45"/>
+      <x:c r="A29" s="73"/>
+      <x:c r="B29" s="73"/>
+      <x:c r="C29" s="73"/>
+      <x:c r="D29" s="73"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="45"/>
-      <x:c r="B30" s="45"/>
-      <x:c r="C30" s="45"/>
-      <x:c r="D30" s="45"/>
+      <x:c r="A30" s="73"/>
+      <x:c r="B30" s="73"/>
+      <x:c r="C30" s="73"/>
+      <x:c r="D30" s="73"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="45"/>
-      <x:c r="B31" s="45"/>
-      <x:c r="C31" s="45"/>
-      <x:c r="D31" s="45"/>
+      <x:c r="A31" s="73"/>
+      <x:c r="B31" s="73"/>
+      <x:c r="C31" s="73"/>
+      <x:c r="D31" s="73"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="45"/>
-      <x:c r="B32" s="45"/>
-      <x:c r="C32" s="45"/>
-      <x:c r="D32" s="45"/>
+      <x:c r="A32" s="73"/>
+      <x:c r="B32" s="73"/>
+      <x:c r="C32" s="73"/>
+      <x:c r="D32" s="73"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="45"/>
-      <x:c r="B33" s="45"/>
-      <x:c r="C33" s="45"/>
-      <x:c r="D33" s="45"/>
+      <x:c r="A33" s="73"/>
+      <x:c r="B33" s="73"/>
+      <x:c r="C33" s="73"/>
+      <x:c r="D33" s="73"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="45"/>
-      <x:c r="B34" s="45"/>
-      <x:c r="C34" s="45"/>
-      <x:c r="D34" s="45"/>
+      <x:c r="A34" s="73"/>
+      <x:c r="B34" s="73"/>
+      <x:c r="C34" s="73"/>
+      <x:c r="D34" s="73"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="45"/>
-      <x:c r="B35" s="45"/>
-      <x:c r="C35" s="45"/>
-      <x:c r="D35" s="45"/>
+      <x:c r="A35" s="73"/>
+      <x:c r="B35" s="73"/>
+      <x:c r="C35" s="73"/>
+      <x:c r="D35" s="73"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="45"/>
-      <x:c r="B36" s="45"/>
-      <x:c r="C36" s="45"/>
-      <x:c r="D36" s="45"/>
+      <x:c r="A36" s="73"/>
+      <x:c r="B36" s="73"/>
+      <x:c r="C36" s="73"/>
+      <x:c r="D36" s="73"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="45"/>
-      <x:c r="B37" s="45"/>
-      <x:c r="C37" s="45"/>
-      <x:c r="D37" s="45"/>
+      <x:c r="A37" s="73"/>
+      <x:c r="B37" s="73"/>
+      <x:c r="C37" s="73"/>
+      <x:c r="D37" s="73"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="45"/>
-      <x:c r="B38" s="45"/>
-      <x:c r="C38" s="45"/>
-      <x:c r="D38" s="45"/>
+      <x:c r="A38" s="73"/>
+      <x:c r="B38" s="73"/>
+      <x:c r="C38" s="73"/>
+      <x:c r="D38" s="73"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="45"/>
-      <x:c r="B39" s="45"/>
-      <x:c r="C39" s="45"/>
-      <x:c r="D39" s="45"/>
+      <x:c r="A39" s="73"/>
+      <x:c r="B39" s="73"/>
+      <x:c r="C39" s="73"/>
+      <x:c r="D39" s="73"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="45"/>
-      <x:c r="B40" s="45"/>
-      <x:c r="C40" s="45"/>
-      <x:c r="D40" s="45"/>
+      <x:c r="A40" s="73"/>
+      <x:c r="B40" s="73"/>
+      <x:c r="C40" s="73"/>
+      <x:c r="D40" s="73"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -2135,12 +3049,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb5cd81d802b4400"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra846efda5ac546ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2154,256 +3068,256 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="71" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Username autista *</x:v>
       </x:c>
-      <x:c r="B1" s="72" t="str">
+      <x:c r="B1" s="82" t="str">
         <x:v>Documento *</x:v>
       </x:c>
-      <x:c r="C1" s="72" t="str">
+      <x:c r="C1" s="82" t="str">
         <x:v>Scadenza documento *</x:v>
       </x:c>
-      <x:c r="D1" s="73" t="str">
+      <x:c r="D1" s="65" t="str">
         <x:v>Numero documento</x:v>
       </x:c>
-      <x:c r="E1" s="73" t="str">
+      <x:c r="E1" s="65" t="str">
         <x:v>Visibile in app</x:v>
       </x:c>
-      <x:c r="F1" s="73" t="str">
+      <x:c r="F1" s="65" t="str">
         <x:v>Responsabile</x:v>
       </x:c>
-      <x:c r="G1" s="74" t="str">
+      <x:c r="G1" s="66" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="87" t="str">
+      <x:c r="A2" s="89" t="str">
         <x:v>mario.rossi</x:v>
       </x:c>
-      <x:c r="B2" s="77" t="str">
+      <x:c r="B2" s="68" t="str">
         <x:v>CQC</x:v>
       </x:c>
-      <x:c r="C2" s="92" t="str">
+      <x:c r="C2" s="94" t="str">
         <x:v>2027-11-30</x:v>
       </x:c>
-      <x:c r="D2" s="76" t="str">
+      <x:c r="D2" s="83" t="str">
         <x:v>CQC9988</x:v>
       </x:c>
-      <x:c r="E2" s="77" t="str">
+      <x:c r="E2" s="68" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="F2" s="77" t="str">
+      <x:c r="F2" s="68" t="str">
         <x:v>Ufficio personale</x:v>
       </x:c>
-      <x:c r="G2" s="78" t="str">
+      <x:c r="G2" s="69" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="88" t="str">
+      <x:c r="A3" s="90" t="str">
         <x:v>anna.verdi</x:v>
       </x:c>
-      <x:c r="B3" s="81" t="str">
+      <x:c r="B3" s="71" t="str">
         <x:v>Visita medica</x:v>
       </x:c>
-      <x:c r="C3" s="93" t="str">
+      <x:c r="C3" s="95" t="str">
         <x:v>2027-04-20</x:v>
       </x:c>
-      <x:c r="D3" s="80" t="str">
+      <x:c r="D3" s="84" t="str">
         <x:v>VM-ANNA</x:v>
       </x:c>
-      <x:c r="E3" s="81" t="str">
+      <x:c r="E3" s="71" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="F3" s="81" t="str">
+      <x:c r="F3" s="71" t="str">
         <x:v>Ufficio personale</x:v>
       </x:c>
-      <x:c r="G3" s="82" t="str"/>
+      <x:c r="G3" s="72" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="45"/>
-      <x:c r="C4" s="94"/>
-      <x:c r="D4" s="45"/>
+      <x:c r="A4" s="73"/>
+      <x:c r="C4" s="96"/>
+      <x:c r="D4" s="73"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="45"/>
-      <x:c r="C5" s="94"/>
-      <x:c r="D5" s="45"/>
+      <x:c r="A5" s="73"/>
+      <x:c r="C5" s="96"/>
+      <x:c r="D5" s="73"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="45"/>
-      <x:c r="C6" s="94"/>
-      <x:c r="D6" s="45"/>
+      <x:c r="A6" s="73"/>
+      <x:c r="C6" s="96"/>
+      <x:c r="D6" s="73"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="45"/>
-      <x:c r="C7" s="94"/>
-      <x:c r="D7" s="45"/>
+      <x:c r="A7" s="73"/>
+      <x:c r="C7" s="96"/>
+      <x:c r="D7" s="73"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="45"/>
-      <x:c r="C8" s="94"/>
-      <x:c r="D8" s="45"/>
+      <x:c r="A8" s="73"/>
+      <x:c r="C8" s="96"/>
+      <x:c r="D8" s="73"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45"/>
-      <x:c r="C9" s="94"/>
-      <x:c r="D9" s="45"/>
+      <x:c r="A9" s="73"/>
+      <x:c r="C9" s="96"/>
+      <x:c r="D9" s="73"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="45"/>
-      <x:c r="C10" s="94"/>
-      <x:c r="D10" s="45"/>
+      <x:c r="A10" s="73"/>
+      <x:c r="C10" s="96"/>
+      <x:c r="D10" s="73"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="45"/>
-      <x:c r="C11" s="94"/>
-      <x:c r="D11" s="45"/>
+      <x:c r="A11" s="73"/>
+      <x:c r="C11" s="96"/>
+      <x:c r="D11" s="73"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="45"/>
-      <x:c r="C12" s="94"/>
-      <x:c r="D12" s="45"/>
+      <x:c r="A12" s="73"/>
+      <x:c r="C12" s="96"/>
+      <x:c r="D12" s="73"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="45"/>
-      <x:c r="C13" s="94"/>
-      <x:c r="D13" s="45"/>
+      <x:c r="A13" s="73"/>
+      <x:c r="C13" s="96"/>
+      <x:c r="D13" s="73"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="45"/>
-      <x:c r="C14" s="94"/>
-      <x:c r="D14" s="45"/>
+      <x:c r="A14" s="73"/>
+      <x:c r="C14" s="96"/>
+      <x:c r="D14" s="73"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="45"/>
-      <x:c r="C15" s="94"/>
-      <x:c r="D15" s="45"/>
+      <x:c r="A15" s="73"/>
+      <x:c r="C15" s="96"/>
+      <x:c r="D15" s="73"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="45"/>
-      <x:c r="C16" s="94"/>
-      <x:c r="D16" s="45"/>
+      <x:c r="A16" s="73"/>
+      <x:c r="C16" s="96"/>
+      <x:c r="D16" s="73"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="45"/>
-      <x:c r="C17" s="94"/>
-      <x:c r="D17" s="45"/>
+      <x:c r="A17" s="73"/>
+      <x:c r="C17" s="96"/>
+      <x:c r="D17" s="73"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="45"/>
-      <x:c r="C18" s="94"/>
-      <x:c r="D18" s="45"/>
+      <x:c r="A18" s="73"/>
+      <x:c r="C18" s="96"/>
+      <x:c r="D18" s="73"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="45"/>
-      <x:c r="C19" s="94"/>
-      <x:c r="D19" s="45"/>
+      <x:c r="A19" s="73"/>
+      <x:c r="C19" s="96"/>
+      <x:c r="D19" s="73"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="45"/>
-      <x:c r="C20" s="94"/>
-      <x:c r="D20" s="45"/>
+      <x:c r="A20" s="73"/>
+      <x:c r="C20" s="96"/>
+      <x:c r="D20" s="73"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="45"/>
-      <x:c r="C21" s="94"/>
-      <x:c r="D21" s="45"/>
+      <x:c r="A21" s="73"/>
+      <x:c r="C21" s="96"/>
+      <x:c r="D21" s="73"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="45"/>
-      <x:c r="C22" s="94"/>
-      <x:c r="D22" s="45"/>
+      <x:c r="A22" s="73"/>
+      <x:c r="C22" s="96"/>
+      <x:c r="D22" s="73"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="45"/>
-      <x:c r="C23" s="94"/>
-      <x:c r="D23" s="45"/>
+      <x:c r="A23" s="73"/>
+      <x:c r="C23" s="96"/>
+      <x:c r="D23" s="73"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="45"/>
-      <x:c r="C24" s="94"/>
-      <x:c r="D24" s="45"/>
+      <x:c r="A24" s="73"/>
+      <x:c r="C24" s="96"/>
+      <x:c r="D24" s="73"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="45"/>
-      <x:c r="C25" s="94"/>
-      <x:c r="D25" s="45"/>
+      <x:c r="A25" s="73"/>
+      <x:c r="C25" s="96"/>
+      <x:c r="D25" s="73"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="45"/>
-      <x:c r="C26" s="94"/>
-      <x:c r="D26" s="45"/>
+      <x:c r="A26" s="73"/>
+      <x:c r="C26" s="96"/>
+      <x:c r="D26" s="73"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="45"/>
-      <x:c r="C27" s="94"/>
-      <x:c r="D27" s="45"/>
+      <x:c r="A27" s="73"/>
+      <x:c r="C27" s="96"/>
+      <x:c r="D27" s="73"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="45"/>
-      <x:c r="C28" s="94"/>
-      <x:c r="D28" s="45"/>
+      <x:c r="A28" s="73"/>
+      <x:c r="C28" s="96"/>
+      <x:c r="D28" s="73"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="45"/>
-      <x:c r="C29" s="94"/>
-      <x:c r="D29" s="45"/>
+      <x:c r="A29" s="73"/>
+      <x:c r="C29" s="96"/>
+      <x:c r="D29" s="73"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="45"/>
-      <x:c r="C30" s="94"/>
-      <x:c r="D30" s="45"/>
+      <x:c r="A30" s="73"/>
+      <x:c r="C30" s="96"/>
+      <x:c r="D30" s="73"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="45"/>
-      <x:c r="C31" s="94"/>
-      <x:c r="D31" s="45"/>
+      <x:c r="A31" s="73"/>
+      <x:c r="C31" s="96"/>
+      <x:c r="D31" s="73"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="45"/>
-      <x:c r="C32" s="94"/>
-      <x:c r="D32" s="45"/>
+      <x:c r="A32" s="73"/>
+      <x:c r="C32" s="96"/>
+      <x:c r="D32" s="73"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="45"/>
-      <x:c r="C33" s="94"/>
-      <x:c r="D33" s="45"/>
+      <x:c r="A33" s="73"/>
+      <x:c r="C33" s="96"/>
+      <x:c r="D33" s="73"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="45"/>
-      <x:c r="C34" s="94"/>
-      <x:c r="D34" s="45"/>
+      <x:c r="A34" s="73"/>
+      <x:c r="C34" s="96"/>
+      <x:c r="D34" s="73"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="45"/>
-      <x:c r="C35" s="94"/>
-      <x:c r="D35" s="45"/>
+      <x:c r="A35" s="73"/>
+      <x:c r="C35" s="96"/>
+      <x:c r="D35" s="73"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="45"/>
-      <x:c r="C36" s="94"/>
-      <x:c r="D36" s="45"/>
+      <x:c r="A36" s="73"/>
+      <x:c r="C36" s="96"/>
+      <x:c r="D36" s="73"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="45"/>
-      <x:c r="C37" s="94"/>
-      <x:c r="D37" s="45"/>
+      <x:c r="A37" s="73"/>
+      <x:c r="C37" s="96"/>
+      <x:c r="D37" s="73"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="45"/>
-      <x:c r="C38" s="94"/>
-      <x:c r="D38" s="45"/>
+      <x:c r="A38" s="73"/>
+      <x:c r="C38" s="96"/>
+      <x:c r="D38" s="73"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="45"/>
-      <x:c r="C39" s="94"/>
-      <x:c r="D39" s="45"/>
+      <x:c r="A39" s="73"/>
+      <x:c r="C39" s="96"/>
+      <x:c r="D39" s="73"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="45"/>
-      <x:c r="C40" s="94"/>
-      <x:c r="D40" s="45"/>
+      <x:c r="A40" s="73"/>
+      <x:c r="C40" s="96"/>
+      <x:c r="D40" s="73"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -2413,12 +3327,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R217f75393eb0412d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91cbc09fc273491a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2433,301 +3347,301 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="71" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Ambito scadenza *</x:v>
       </x:c>
-      <x:c r="B1" s="72" t="str">
+      <x:c r="B1" s="82" t="str">
         <x:v>Username o targa o codice *</x:v>
       </x:c>
-      <x:c r="C1" s="72" t="str">
+      <x:c r="C1" s="82" t="str">
         <x:v>Tipo scadenza *</x:v>
       </x:c>
-      <x:c r="D1" s="72" t="str">
+      <x:c r="D1" s="82" t="str">
         <x:v>Data scadenza *</x:v>
       </x:c>
-      <x:c r="E1" s="73" t="str">
+      <x:c r="E1" s="65" t="str">
         <x:v>Numero documento</x:v>
       </x:c>
-      <x:c r="F1" s="73" t="str">
+      <x:c r="F1" s="65" t="str">
         <x:v>Responsabile</x:v>
       </x:c>
-      <x:c r="G1" s="73" t="str">
+      <x:c r="G1" s="65" t="str">
         <x:v>Visibile in app</x:v>
       </x:c>
-      <x:c r="H1" s="74" t="str">
+      <x:c r="H1" s="66" t="str">
         <x:v>Note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="75" t="str">
+      <x:c r="A2" s="67" t="str">
         <x:v>mezzo</x:v>
       </x:c>
-      <x:c r="B2" s="76" t="str">
+      <x:c r="B2" s="83" t="str">
         <x:v>AB123CD</x:v>
       </x:c>
-      <x:c r="C2" s="77" t="str">
+      <x:c r="C2" s="68" t="str">
         <x:v>Revisione mezzo</x:v>
       </x:c>
-      <x:c r="D2" s="92" t="str">
+      <x:c r="D2" s="94" t="str">
         <x:v>2026-12-15</x:v>
       </x:c>
-      <x:c r="E2" s="76" t="str">
+      <x:c r="E2" s="83" t="str">
         <x:v>REV-AB123CD</x:v>
       </x:c>
-      <x:c r="F2" s="77" t="str">
+      <x:c r="F2" s="68" t="str">
         <x:v>Ufficio flotta</x:v>
       </x:c>
-      <x:c r="G2" s="77" t="str">
+      <x:c r="G2" s="68" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="H2" s="78" t="str">
+      <x:c r="H2" s="69" t="str">
         <x:v>Riga esempio: puoi cancellarla</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="75" t="str">
+      <x:c r="A3" s="67" t="str">
         <x:v>attrezzatura</x:v>
       </x:c>
-      <x:c r="B3" s="76" t="str">
+      <x:c r="B3" s="83" t="str">
         <x:v>MUL-01</x:v>
       </x:c>
-      <x:c r="C3" s="77" t="str">
+      <x:c r="C3" s="68" t="str">
         <x:v>Verifica sicurezza muletto</x:v>
       </x:c>
-      <x:c r="D3" s="92" t="str">
+      <x:c r="D3" s="94" t="str">
         <x:v>2026-10-10</x:v>
       </x:c>
-      <x:c r="E3" s="76" t="str">
+      <x:c r="E3" s="83" t="str">
         <x:v>CHK-MUL01</x:v>
       </x:c>
-      <x:c r="F3" s="77" t="str">
+      <x:c r="F3" s="68" t="str">
         <x:v>Responsabile magazzino</x:v>
       </x:c>
-      <x:c r="G3" s="77" t="str">
+      <x:c r="G3" s="68" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="H3" s="78" t="str"/>
+      <x:c r="H3" s="69" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="75" t="str">
+      <x:c r="A4" s="67" t="str">
         <x:v>persona</x:v>
       </x:c>
-      <x:c r="B4" s="76" t="str">
+      <x:c r="B4" s="83" t="str">
         <x:v>luca.neri</x:v>
       </x:c>
-      <x:c r="C4" s="77" t="str">
+      <x:c r="C4" s="68" t="str">
         <x:v>Visita medica</x:v>
       </x:c>
-      <x:c r="D4" s="92" t="str">
+      <x:c r="D4" s="94" t="str">
         <x:v>2027-02-01</x:v>
       </x:c>
-      <x:c r="E4" s="76" t="str">
+      <x:c r="E4" s="83" t="str">
         <x:v>VM-LUCA</x:v>
       </x:c>
-      <x:c r="F4" s="77" t="str">
+      <x:c r="F4" s="68" t="str">
         <x:v>Ufficio personale</x:v>
       </x:c>
-      <x:c r="G4" s="77" t="str">
+      <x:c r="G4" s="68" t="str">
         <x:v>si</x:v>
       </x:c>
-      <x:c r="H4" s="78" t="str"/>
+      <x:c r="H4" s="69" t="str"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="79" t="str">
+      <x:c r="A5" s="70" t="str">
         <x:v>azienda</x:v>
       </x:c>
-      <x:c r="B5" s="80" t="str"/>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="B5" s="84" t="str"/>
+      <x:c r="C5" s="71" t="str">
         <x:v>Polizza sede</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="95" t="str">
         <x:v>2027-01-31</x:v>
       </x:c>
-      <x:c r="E5" s="80" t="str">
+      <x:c r="E5" s="84" t="str">
         <x:v>POL-SEDE</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="71" t="str">
         <x:v>Amministrazione</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="71" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="H5" s="82" t="str"/>
+      <x:c r="H5" s="72" t="str"/>
     </x:row>
     <x:row r="6">
-      <x:c r="B6" s="45"/>
-      <x:c r="D6" s="94"/>
-      <x:c r="E6" s="45"/>
+      <x:c r="B6" s="73"/>
+      <x:c r="D6" s="96"/>
+      <x:c r="E6" s="73"/>
     </x:row>
     <x:row r="7">
-      <x:c r="B7" s="45"/>
-      <x:c r="D7" s="94"/>
-      <x:c r="E7" s="45"/>
+      <x:c r="B7" s="73"/>
+      <x:c r="D7" s="96"/>
+      <x:c r="E7" s="73"/>
     </x:row>
     <x:row r="8">
-      <x:c r="B8" s="45"/>
-      <x:c r="D8" s="94"/>
-      <x:c r="E8" s="45"/>
+      <x:c r="B8" s="73"/>
+      <x:c r="D8" s="96"/>
+      <x:c r="E8" s="73"/>
     </x:row>
     <x:row r="9">
-      <x:c r="B9" s="45"/>
-      <x:c r="D9" s="94"/>
-      <x:c r="E9" s="45"/>
+      <x:c r="B9" s="73"/>
+      <x:c r="D9" s="96"/>
+      <x:c r="E9" s="73"/>
     </x:row>
     <x:row r="10">
-      <x:c r="B10" s="45"/>
-      <x:c r="D10" s="94"/>
-      <x:c r="E10" s="45"/>
+      <x:c r="B10" s="73"/>
+      <x:c r="D10" s="96"/>
+      <x:c r="E10" s="73"/>
     </x:row>
     <x:row r="11">
-      <x:c r="B11" s="45"/>
-      <x:c r="D11" s="94"/>
-      <x:c r="E11" s="45"/>
+      <x:c r="B11" s="73"/>
+      <x:c r="D11" s="96"/>
+      <x:c r="E11" s="73"/>
     </x:row>
     <x:row r="12">
-      <x:c r="B12" s="45"/>
-      <x:c r="D12" s="94"/>
-      <x:c r="E12" s="45"/>
+      <x:c r="B12" s="73"/>
+      <x:c r="D12" s="96"/>
+      <x:c r="E12" s="73"/>
     </x:row>
     <x:row r="13">
-      <x:c r="B13" s="45"/>
-      <x:c r="D13" s="94"/>
-      <x:c r="E13" s="45"/>
+      <x:c r="B13" s="73"/>
+      <x:c r="D13" s="96"/>
+      <x:c r="E13" s="73"/>
     </x:row>
     <x:row r="14">
-      <x:c r="B14" s="45"/>
-      <x:c r="D14" s="94"/>
-      <x:c r="E14" s="45"/>
+      <x:c r="B14" s="73"/>
+      <x:c r="D14" s="96"/>
+      <x:c r="E14" s="73"/>
     </x:row>
     <x:row r="15">
-      <x:c r="B15" s="45"/>
-      <x:c r="D15" s="94"/>
-      <x:c r="E15" s="45"/>
+      <x:c r="B15" s="73"/>
+      <x:c r="D15" s="96"/>
+      <x:c r="E15" s="73"/>
     </x:row>
     <x:row r="16">
-      <x:c r="B16" s="45"/>
-      <x:c r="D16" s="94"/>
-      <x:c r="E16" s="45"/>
+      <x:c r="B16" s="73"/>
+      <x:c r="D16" s="96"/>
+      <x:c r="E16" s="73"/>
     </x:row>
     <x:row r="17">
-      <x:c r="B17" s="45"/>
-      <x:c r="D17" s="94"/>
-      <x:c r="E17" s="45"/>
+      <x:c r="B17" s="73"/>
+      <x:c r="D17" s="96"/>
+      <x:c r="E17" s="73"/>
     </x:row>
     <x:row r="18">
-      <x:c r="B18" s="45"/>
-      <x:c r="D18" s="94"/>
-      <x:c r="E18" s="45"/>
+      <x:c r="B18" s="73"/>
+      <x:c r="D18" s="96"/>
+      <x:c r="E18" s="73"/>
     </x:row>
     <x:row r="19">
-      <x:c r="B19" s="45"/>
-      <x:c r="D19" s="94"/>
-      <x:c r="E19" s="45"/>
+      <x:c r="B19" s="73"/>
+      <x:c r="D19" s="96"/>
+      <x:c r="E19" s="73"/>
     </x:row>
     <x:row r="20">
-      <x:c r="B20" s="45"/>
-      <x:c r="D20" s="94"/>
-      <x:c r="E20" s="45"/>
+      <x:c r="B20" s="73"/>
+      <x:c r="D20" s="96"/>
+      <x:c r="E20" s="73"/>
     </x:row>
     <x:row r="21">
-      <x:c r="B21" s="45"/>
-      <x:c r="D21" s="94"/>
-      <x:c r="E21" s="45"/>
+      <x:c r="B21" s="73"/>
+      <x:c r="D21" s="96"/>
+      <x:c r="E21" s="73"/>
     </x:row>
     <x:row r="22">
-      <x:c r="B22" s="45"/>
-      <x:c r="D22" s="94"/>
-      <x:c r="E22" s="45"/>
+      <x:c r="B22" s="73"/>
+      <x:c r="D22" s="96"/>
+      <x:c r="E22" s="73"/>
     </x:row>
     <x:row r="23">
-      <x:c r="B23" s="45"/>
-      <x:c r="D23" s="94"/>
-      <x:c r="E23" s="45"/>
+      <x:c r="B23" s="73"/>
+      <x:c r="D23" s="96"/>
+      <x:c r="E23" s="73"/>
     </x:row>
     <x:row r="24">
-      <x:c r="B24" s="45"/>
-      <x:c r="D24" s="94"/>
-      <x:c r="E24" s="45"/>
+      <x:c r="B24" s="73"/>
+      <x:c r="D24" s="96"/>
+      <x:c r="E24" s="73"/>
     </x:row>
     <x:row r="25">
-      <x:c r="B25" s="45"/>
-      <x:c r="D25" s="94"/>
-      <x:c r="E25" s="45"/>
+      <x:c r="B25" s="73"/>
+      <x:c r="D25" s="96"/>
+      <x:c r="E25" s="73"/>
     </x:row>
     <x:row r="26">
-      <x:c r="B26" s="45"/>
-      <x:c r="D26" s="94"/>
-      <x:c r="E26" s="45"/>
+      <x:c r="B26" s="73"/>
+      <x:c r="D26" s="96"/>
+      <x:c r="E26" s="73"/>
     </x:row>
     <x:row r="27">
-      <x:c r="B27" s="45"/>
-      <x:c r="D27" s="94"/>
-      <x:c r="E27" s="45"/>
+      <x:c r="B27" s="73"/>
+      <x:c r="D27" s="96"/>
+      <x:c r="E27" s="73"/>
     </x:row>
     <x:row r="28">
-      <x:c r="B28" s="45"/>
-      <x:c r="D28" s="94"/>
-      <x:c r="E28" s="45"/>
+      <x:c r="B28" s="73"/>
+      <x:c r="D28" s="96"/>
+      <x:c r="E28" s="73"/>
     </x:row>
     <x:row r="29">
-      <x:c r="B29" s="45"/>
-      <x:c r="D29" s="94"/>
-      <x:c r="E29" s="45"/>
+      <x:c r="B29" s="73"/>
+      <x:c r="D29" s="96"/>
+      <x:c r="E29" s="73"/>
     </x:row>
     <x:row r="30">
-      <x:c r="B30" s="45"/>
-      <x:c r="D30" s="94"/>
-      <x:c r="E30" s="45"/>
+      <x:c r="B30" s="73"/>
+      <x:c r="D30" s="96"/>
+      <x:c r="E30" s="73"/>
     </x:row>
     <x:row r="31">
-      <x:c r="B31" s="45"/>
-      <x:c r="D31" s="94"/>
-      <x:c r="E31" s="45"/>
+      <x:c r="B31" s="73"/>
+      <x:c r="D31" s="96"/>
+      <x:c r="E31" s="73"/>
     </x:row>
     <x:row r="32">
-      <x:c r="B32" s="45"/>
-      <x:c r="D32" s="94"/>
-      <x:c r="E32" s="45"/>
+      <x:c r="B32" s="73"/>
+      <x:c r="D32" s="96"/>
+      <x:c r="E32" s="73"/>
     </x:row>
     <x:row r="33">
-      <x:c r="B33" s="45"/>
-      <x:c r="D33" s="94"/>
-      <x:c r="E33" s="45"/>
+      <x:c r="B33" s="73"/>
+      <x:c r="D33" s="96"/>
+      <x:c r="E33" s="73"/>
     </x:row>
     <x:row r="34">
-      <x:c r="B34" s="45"/>
-      <x:c r="D34" s="94"/>
-      <x:c r="E34" s="45"/>
+      <x:c r="B34" s="73"/>
+      <x:c r="D34" s="96"/>
+      <x:c r="E34" s="73"/>
     </x:row>
     <x:row r="35">
-      <x:c r="B35" s="45"/>
-      <x:c r="D35" s="94"/>
-      <x:c r="E35" s="45"/>
+      <x:c r="B35" s="73"/>
+      <x:c r="D35" s="96"/>
+      <x:c r="E35" s="73"/>
     </x:row>
     <x:row r="36">
-      <x:c r="B36" s="45"/>
-      <x:c r="D36" s="94"/>
-      <x:c r="E36" s="45"/>
+      <x:c r="B36" s="73"/>
+      <x:c r="D36" s="96"/>
+      <x:c r="E36" s="73"/>
     </x:row>
     <x:row r="37">
-      <x:c r="B37" s="45"/>
-      <x:c r="D37" s="94"/>
-      <x:c r="E37" s="45"/>
+      <x:c r="B37" s="73"/>
+      <x:c r="D37" s="96"/>
+      <x:c r="E37" s="73"/>
     </x:row>
     <x:row r="38">
-      <x:c r="B38" s="45"/>
-      <x:c r="D38" s="94"/>
-      <x:c r="E38" s="45"/>
+      <x:c r="B38" s="73"/>
+      <x:c r="D38" s="96"/>
+      <x:c r="E38" s="73"/>
     </x:row>
     <x:row r="39">
-      <x:c r="B39" s="45"/>
-      <x:c r="D39" s="94"/>
-      <x:c r="E39" s="45"/>
+      <x:c r="B39" s="73"/>
+      <x:c r="D39" s="96"/>
+      <x:c r="E39" s="73"/>
     </x:row>
     <x:row r="40">
-      <x:c r="B40" s="45"/>
-      <x:c r="D40" s="94"/>
-      <x:c r="E40" s="45"/>
+      <x:c r="B40" s="73"/>
+      <x:c r="D40" s="96"/>
+      <x:c r="E40" s="73"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -2740,7 +3654,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfa97270ca0a43c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c99b149cb4e4192"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>